<commit_message>
Seguimiento front y schema
</commit_message>
<xml_diff>
--- a/backend/TestEjemplo - copia.xlsx
+++ b/backend/TestEjemplo - copia.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fiduprevisora-my.sharepoint.com/personal/p_scorrea_fiduprevisora_com_co/Documents/Escritorio/contratos-dashboard/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="8_{4CA17712-2CC0-4CCD-AA75-F19B91EB8E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6C6B920E-AA4F-492C-B714-1E4DAA5C59BE}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="8_{4CA17712-2CC0-4CCD-AA75-F19B91EB8E68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{76ED143C-24ED-4D5F-93C0-D6608796E5AD}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -395,7 +395,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="153">
   <si>
     <t>I.- GENERALIDADES DEL CONTRATO</t>
   </si>
@@ -936,13 +936,7 @@
     <t>Fecha:</t>
   </si>
   <si>
-    <t>1-9000-145-2025</t>
-  </si>
-  <si>
     <t>PRESTACION DE SERVICIOS</t>
-  </si>
-  <si>
-    <t>JUAN ANTONIO URIBE DE SATORY</t>
   </si>
   <si>
     <t>El CONTRATISTA con autonomía técnica y administrativa, se obliga con el CONTRATANTE a prestar los servicios de soporte, actualización y mantenimiento del aplicativo MITRA y la plataforma JAC versión ONPREMISE ESTANDAR, como también migración, implementación, soporte, actualización y mantenimiento del aplicativo MITRA Clúster SaaS, los cuales permiten realizar la integración entre el aplicativo MITRA y la Bolsa de Valores de Colombia. Lo anterior, de conformidad con la propuesta presentada por el CONTRATISTA, la cual hace parte integral del presente CONTRATO, en lo que no contravenga las disposiciones pactadas en el mismo.</t>
@@ -1108,7 +1102,16 @@
     <t>18 meses</t>
   </si>
   <si>
-    <t>JUAN ANDRES PEREIRA</t>
+    <t>5 meses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SEBASTIAN </t>
+  </si>
+  <si>
+    <t>Esteban Suarez</t>
+  </si>
+  <si>
+    <t>1-9000-133-2025</t>
   </si>
 </sst>
 </file>
@@ -2444,7 +2447,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="29" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="418">
+  <cellXfs count="419">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3136,6 +3139,9 @@
     <xf numFmtId="15" fontId="4" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="15" fontId="31" fillId="5" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="15" fontId="4" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3306,6 +3312,9 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="5" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3316,9 +3325,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="5" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="34" fillId="5" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4205,53 +4211,53 @@
       <c r="G2" s="17"/>
       <c r="H2" s="17"/>
       <c r="I2" s="17"/>
-      <c r="J2" s="289" t="s">
+      <c r="J2" s="290" t="s">
         <v>56</v>
       </c>
-      <c r="K2" s="289"/>
-      <c r="L2" s="289"/>
-      <c r="M2" s="289"/>
-      <c r="N2" s="289"/>
-      <c r="O2" s="289"/>
-      <c r="P2" s="289"/>
-      <c r="Q2" s="289"/>
-      <c r="R2" s="289"/>
-      <c r="S2" s="289"/>
-      <c r="T2" s="289"/>
-      <c r="U2" s="289"/>
-      <c r="V2" s="289"/>
-      <c r="W2" s="289"/>
-      <c r="X2" s="289"/>
-      <c r="Y2" s="289"/>
-      <c r="Z2" s="289"/>
-      <c r="AA2" s="289"/>
-      <c r="AB2" s="289"/>
-      <c r="AC2" s="289"/>
-      <c r="AD2" s="289"/>
-      <c r="AE2" s="289"/>
-      <c r="AF2" s="289"/>
-      <c r="AG2" s="289"/>
-      <c r="AH2" s="289"/>
-      <c r="AI2" s="289"/>
-      <c r="AJ2" s="289"/>
-      <c r="AK2" s="289"/>
+      <c r="K2" s="290"/>
+      <c r="L2" s="290"/>
+      <c r="M2" s="290"/>
+      <c r="N2" s="290"/>
+      <c r="O2" s="290"/>
+      <c r="P2" s="290"/>
+      <c r="Q2" s="290"/>
+      <c r="R2" s="290"/>
+      <c r="S2" s="290"/>
+      <c r="T2" s="290"/>
+      <c r="U2" s="290"/>
+      <c r="V2" s="290"/>
+      <c r="W2" s="290"/>
+      <c r="X2" s="290"/>
+      <c r="Y2" s="290"/>
+      <c r="Z2" s="290"/>
+      <c r="AA2" s="290"/>
+      <c r="AB2" s="290"/>
+      <c r="AC2" s="290"/>
+      <c r="AD2" s="290"/>
+      <c r="AE2" s="290"/>
+      <c r="AF2" s="290"/>
+      <c r="AG2" s="290"/>
+      <c r="AH2" s="290"/>
+      <c r="AI2" s="290"/>
+      <c r="AJ2" s="290"/>
+      <c r="AK2" s="290"/>
       <c r="AL2" s="36"/>
       <c r="AM2" s="17"/>
       <c r="AN2" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="AO2" s="281">
+      <c r="AO2" s="282">
         <v>16</v>
       </c>
-      <c r="AP2" s="282"/>
-      <c r="AQ2" s="278">
+      <c r="AP2" s="283"/>
+      <c r="AQ2" s="279">
         <v>1</v>
       </c>
-      <c r="AR2" s="280"/>
-      <c r="AS2" s="278">
+      <c r="AR2" s="281"/>
+      <c r="AS2" s="279">
         <v>2026</v>
       </c>
-      <c r="AT2" s="279"/>
+      <c r="AT2" s="280"/>
       <c r="AU2" s="14"/>
     </row>
     <row r="3" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -4264,34 +4270,34 @@
       <c r="G3" s="17"/>
       <c r="H3" s="17"/>
       <c r="I3" s="17"/>
-      <c r="J3" s="289"/>
-      <c r="K3" s="289"/>
-      <c r="L3" s="289"/>
-      <c r="M3" s="289"/>
-      <c r="N3" s="289"/>
-      <c r="O3" s="289"/>
-      <c r="P3" s="289"/>
-      <c r="Q3" s="289"/>
-      <c r="R3" s="289"/>
-      <c r="S3" s="289"/>
-      <c r="T3" s="289"/>
-      <c r="U3" s="289"/>
-      <c r="V3" s="289"/>
-      <c r="W3" s="289"/>
-      <c r="X3" s="289"/>
-      <c r="Y3" s="289"/>
-      <c r="Z3" s="289"/>
-      <c r="AA3" s="289"/>
-      <c r="AB3" s="289"/>
-      <c r="AC3" s="289"/>
-      <c r="AD3" s="289"/>
-      <c r="AE3" s="289"/>
-      <c r="AF3" s="289"/>
-      <c r="AG3" s="289"/>
-      <c r="AH3" s="289"/>
-      <c r="AI3" s="289"/>
-      <c r="AJ3" s="289"/>
-      <c r="AK3" s="289"/>
+      <c r="J3" s="290"/>
+      <c r="K3" s="290"/>
+      <c r="L3" s="290"/>
+      <c r="M3" s="290"/>
+      <c r="N3" s="290"/>
+      <c r="O3" s="290"/>
+      <c r="P3" s="290"/>
+      <c r="Q3" s="290"/>
+      <c r="R3" s="290"/>
+      <c r="S3" s="290"/>
+      <c r="T3" s="290"/>
+      <c r="U3" s="290"/>
+      <c r="V3" s="290"/>
+      <c r="W3" s="290"/>
+      <c r="X3" s="290"/>
+      <c r="Y3" s="290"/>
+      <c r="Z3" s="290"/>
+      <c r="AA3" s="290"/>
+      <c r="AB3" s="290"/>
+      <c r="AC3" s="290"/>
+      <c r="AD3" s="290"/>
+      <c r="AE3" s="290"/>
+      <c r="AF3" s="290"/>
+      <c r="AG3" s="290"/>
+      <c r="AH3" s="290"/>
+      <c r="AI3" s="290"/>
+      <c r="AJ3" s="290"/>
+      <c r="AK3" s="290"/>
       <c r="AL3" s="17"/>
       <c r="AM3" s="17"/>
       <c r="AN3" s="26"/>
@@ -4454,151 +4460,151 @@
     </row>
     <row r="7" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="59"/>
-      <c r="B7" s="290" t="s">
+      <c r="B7" s="291" t="s">
         <v>57</v>
       </c>
-      <c r="C7" s="290"/>
-      <c r="D7" s="290"/>
-      <c r="E7" s="290"/>
-      <c r="F7" s="290"/>
-      <c r="G7" s="290"/>
-      <c r="H7" s="290"/>
-      <c r="I7" s="288" t="s">
-        <v>141</v>
-      </c>
-      <c r="J7" s="288"/>
-      <c r="K7" s="288"/>
-      <c r="L7" s="288"/>
-      <c r="M7" s="288"/>
-      <c r="N7" s="288"/>
-      <c r="O7" s="288"/>
-      <c r="P7" s="288"/>
-      <c r="Q7" s="288"/>
-      <c r="R7" s="288"/>
-      <c r="S7" s="288"/>
-      <c r="T7" s="288"/>
-      <c r="U7" s="288"/>
-      <c r="V7" s="288"/>
-      <c r="W7" s="288"/>
-      <c r="X7" s="288"/>
-      <c r="Y7" s="288"/>
-      <c r="Z7" s="288"/>
-      <c r="AA7" s="288"/>
-      <c r="AB7" s="288"/>
+      <c r="C7" s="291"/>
+      <c r="D7" s="291"/>
+      <c r="E7" s="291"/>
+      <c r="F7" s="291"/>
+      <c r="G7" s="291"/>
+      <c r="H7" s="291"/>
+      <c r="I7" s="289" t="s">
+        <v>139</v>
+      </c>
+      <c r="J7" s="289"/>
+      <c r="K7" s="289"/>
+      <c r="L7" s="289"/>
+      <c r="M7" s="289"/>
+      <c r="N7" s="289"/>
+      <c r="O7" s="289"/>
+      <c r="P7" s="289"/>
+      <c r="Q7" s="289"/>
+      <c r="R7" s="289"/>
+      <c r="S7" s="289"/>
+      <c r="T7" s="289"/>
+      <c r="U7" s="289"/>
+      <c r="V7" s="289"/>
+      <c r="W7" s="289"/>
+      <c r="X7" s="289"/>
+      <c r="Y7" s="289"/>
+      <c r="Z7" s="289"/>
+      <c r="AA7" s="289"/>
+      <c r="AB7" s="289"/>
       <c r="AC7" s="61"/>
-      <c r="AD7" s="290" t="s">
+      <c r="AD7" s="291" t="s">
         <v>5</v>
       </c>
-      <c r="AE7" s="290"/>
-      <c r="AF7" s="290"/>
-      <c r="AG7" s="290"/>
-      <c r="AH7" s="290"/>
-      <c r="AI7" s="290"/>
-      <c r="AJ7" s="290"/>
-      <c r="AK7" s="285" t="s">
-        <v>142</v>
-      </c>
-      <c r="AL7" s="285"/>
-      <c r="AM7" s="285"/>
-      <c r="AN7" s="285"/>
-      <c r="AO7" s="285"/>
-      <c r="AP7" s="285"/>
-      <c r="AQ7" s="285"/>
-      <c r="AR7" s="285"/>
-      <c r="AS7" s="285"/>
-      <c r="AT7" s="285"/>
+      <c r="AE7" s="291"/>
+      <c r="AF7" s="291"/>
+      <c r="AG7" s="291"/>
+      <c r="AH7" s="291"/>
+      <c r="AI7" s="291"/>
+      <c r="AJ7" s="291"/>
+      <c r="AK7" s="286" t="s">
+        <v>140</v>
+      </c>
+      <c r="AL7" s="286"/>
+      <c r="AM7" s="286"/>
+      <c r="AN7" s="286"/>
+      <c r="AO7" s="286"/>
+      <c r="AP7" s="286"/>
+      <c r="AQ7" s="286"/>
+      <c r="AR7" s="286"/>
+      <c r="AS7" s="286"/>
+      <c r="AT7" s="286"/>
       <c r="AU7" s="62"/>
     </row>
     <row r="8" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="59"/>
-      <c r="B8" s="290" t="s">
+      <c r="B8" s="291" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="290"/>
-      <c r="D8" s="290"/>
-      <c r="E8" s="290"/>
-      <c r="F8" s="290"/>
-      <c r="G8" s="290"/>
-      <c r="H8" s="290"/>
-      <c r="I8" s="288" t="s">
+      <c r="C8" s="291"/>
+      <c r="D8" s="291"/>
+      <c r="E8" s="291"/>
+      <c r="F8" s="291"/>
+      <c r="G8" s="291"/>
+      <c r="H8" s="291"/>
+      <c r="I8" s="289" t="s">
+        <v>152</v>
+      </c>
+      <c r="J8" s="289"/>
+      <c r="K8" s="289"/>
+      <c r="L8" s="289"/>
+      <c r="M8" s="289"/>
+      <c r="N8" s="289"/>
+      <c r="O8" s="289"/>
+      <c r="P8" s="289"/>
+      <c r="Q8" s="289"/>
+      <c r="R8" s="289"/>
+      <c r="S8" s="289"/>
+      <c r="T8" s="289"/>
+      <c r="U8" s="289"/>
+      <c r="V8" s="289"/>
+      <c r="W8" s="289"/>
+      <c r="X8" s="289"/>
+      <c r="Y8" s="289"/>
+      <c r="Z8" s="289"/>
+      <c r="AA8" s="289"/>
+      <c r="AB8" s="289"/>
+      <c r="AC8" s="64"/>
+      <c r="AD8" s="287" t="s">
+        <v>73</v>
+      </c>
+      <c r="AE8" s="287"/>
+      <c r="AF8" s="287"/>
+      <c r="AG8" s="287"/>
+      <c r="AH8" s="287"/>
+      <c r="AI8" s="287"/>
+      <c r="AJ8" s="288"/>
+      <c r="AK8" s="284" t="s">
         <v>102</v>
       </c>
-      <c r="J8" s="288"/>
-      <c r="K8" s="288"/>
-      <c r="L8" s="288"/>
-      <c r="M8" s="288"/>
-      <c r="N8" s="288"/>
-      <c r="O8" s="288"/>
-      <c r="P8" s="288"/>
-      <c r="Q8" s="288"/>
-      <c r="R8" s="288"/>
-      <c r="S8" s="288"/>
-      <c r="T8" s="288"/>
-      <c r="U8" s="288"/>
-      <c r="V8" s="288"/>
-      <c r="W8" s="288"/>
-      <c r="X8" s="288"/>
-      <c r="Y8" s="288"/>
-      <c r="Z8" s="288"/>
-      <c r="AA8" s="288"/>
-      <c r="AB8" s="288"/>
-      <c r="AC8" s="64"/>
-      <c r="AD8" s="286" t="s">
-        <v>73</v>
-      </c>
-      <c r="AE8" s="286"/>
-      <c r="AF8" s="286"/>
-      <c r="AG8" s="286"/>
-      <c r="AH8" s="286"/>
-      <c r="AI8" s="286"/>
-      <c r="AJ8" s="287"/>
-      <c r="AK8" s="283" t="s">
-        <v>103</v>
-      </c>
-      <c r="AL8" s="283"/>
-      <c r="AM8" s="283"/>
-      <c r="AN8" s="283"/>
-      <c r="AO8" s="283"/>
-      <c r="AP8" s="283"/>
-      <c r="AQ8" s="283"/>
-      <c r="AR8" s="283"/>
-      <c r="AS8" s="283"/>
-      <c r="AT8" s="284"/>
+      <c r="AL8" s="284"/>
+      <c r="AM8" s="284"/>
+      <c r="AN8" s="284"/>
+      <c r="AO8" s="284"/>
+      <c r="AP8" s="284"/>
+      <c r="AQ8" s="284"/>
+      <c r="AR8" s="284"/>
+      <c r="AS8" s="284"/>
+      <c r="AT8" s="285"/>
       <c r="AU8" s="62"/>
     </row>
     <row r="9" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="59"/>
-      <c r="B9" s="290" t="s">
+      <c r="B9" s="291" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="290"/>
-      <c r="D9" s="290"/>
-      <c r="E9" s="290"/>
-      <c r="F9" s="290"/>
-      <c r="G9" s="290"/>
-      <c r="H9" s="290"/>
-      <c r="I9" s="288" t="s">
-        <v>151</v>
-      </c>
-      <c r="J9" s="288"/>
-      <c r="K9" s="288"/>
-      <c r="L9" s="288"/>
-      <c r="M9" s="288"/>
-      <c r="N9" s="288"/>
-      <c r="O9" s="288"/>
-      <c r="P9" s="288"/>
-      <c r="Q9" s="288"/>
-      <c r="R9" s="288"/>
-      <c r="S9" s="288"/>
-      <c r="T9" s="288"/>
-      <c r="U9" s="288"/>
-      <c r="V9" s="288"/>
-      <c r="W9" s="288"/>
-      <c r="X9" s="288"/>
-      <c r="Y9" s="288"/>
-      <c r="Z9" s="288"/>
-      <c r="AA9" s="288"/>
-      <c r="AB9" s="288"/>
+      <c r="C9" s="291"/>
+      <c r="D9" s="291"/>
+      <c r="E9" s="291"/>
+      <c r="F9" s="291"/>
+      <c r="G9" s="291"/>
+      <c r="H9" s="291"/>
+      <c r="I9" s="292" t="s">
+        <v>150</v>
+      </c>
+      <c r="J9" s="292"/>
+      <c r="K9" s="292"/>
+      <c r="L9" s="292"/>
+      <c r="M9" s="292"/>
+      <c r="N9" s="292"/>
+      <c r="O9" s="292"/>
+      <c r="P9" s="292"/>
+      <c r="Q9" s="292"/>
+      <c r="R9" s="292"/>
+      <c r="S9" s="292"/>
+      <c r="T9" s="292"/>
+      <c r="U9" s="292"/>
+      <c r="V9" s="292"/>
+      <c r="W9" s="292"/>
+      <c r="X9" s="292"/>
+      <c r="Y9" s="292"/>
+      <c r="Z9" s="292"/>
+      <c r="AA9" s="292"/>
+      <c r="AB9" s="292"/>
       <c r="AC9" s="64"/>
       <c r="AD9" s="65" t="s">
         <v>34</v>
@@ -4611,57 +4617,57 @@
       <c r="AH9" s="66" t="s">
         <v>100</v>
       </c>
-      <c r="AI9" s="293" t="s">
+      <c r="AI9" s="295" t="s">
         <v>3</v>
       </c>
-      <c r="AJ9" s="294"/>
-      <c r="AK9" s="291">
+      <c r="AJ9" s="296"/>
+      <c r="AK9" s="293">
         <v>1014015918</v>
       </c>
-      <c r="AL9" s="291"/>
-      <c r="AM9" s="291"/>
-      <c r="AN9" s="291"/>
-      <c r="AO9" s="291"/>
-      <c r="AP9" s="291"/>
-      <c r="AQ9" s="291"/>
-      <c r="AR9" s="291"/>
-      <c r="AS9" s="291"/>
-      <c r="AT9" s="292"/>
+      <c r="AL9" s="293"/>
+      <c r="AM9" s="293"/>
+      <c r="AN9" s="293"/>
+      <c r="AO9" s="293"/>
+      <c r="AP9" s="293"/>
+      <c r="AQ9" s="293"/>
+      <c r="AR9" s="293"/>
+      <c r="AS9" s="293"/>
+      <c r="AT9" s="294"/>
       <c r="AU9" s="62"/>
     </row>
     <row r="10" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="59"/>
-      <c r="B10" s="290" t="s">
+      <c r="B10" s="291" t="s">
         <v>4</v>
       </c>
-      <c r="C10" s="290"/>
-      <c r="D10" s="290"/>
-      <c r="E10" s="290"/>
-      <c r="F10" s="290"/>
-      <c r="G10" s="290"/>
-      <c r="H10" s="290"/>
-      <c r="I10" s="295" t="s">
-        <v>104</v>
-      </c>
-      <c r="J10" s="295"/>
-      <c r="K10" s="295"/>
-      <c r="L10" s="295"/>
-      <c r="M10" s="295"/>
-      <c r="N10" s="295"/>
-      <c r="O10" s="295"/>
-      <c r="P10" s="295"/>
-      <c r="Q10" s="295"/>
-      <c r="R10" s="295"/>
-      <c r="S10" s="295"/>
-      <c r="T10" s="295"/>
-      <c r="U10" s="295"/>
-      <c r="V10" s="295"/>
-      <c r="W10" s="295"/>
-      <c r="X10" s="295"/>
-      <c r="Y10" s="295"/>
-      <c r="Z10" s="295"/>
-      <c r="AA10" s="295"/>
-      <c r="AB10" s="295"/>
+      <c r="C10" s="291"/>
+      <c r="D10" s="291"/>
+      <c r="E10" s="291"/>
+      <c r="F10" s="291"/>
+      <c r="G10" s="291"/>
+      <c r="H10" s="291"/>
+      <c r="I10" s="289" t="s">
+        <v>151</v>
+      </c>
+      <c r="J10" s="289"/>
+      <c r="K10" s="289"/>
+      <c r="L10" s="289"/>
+      <c r="M10" s="289"/>
+      <c r="N10" s="289"/>
+      <c r="O10" s="289"/>
+      <c r="P10" s="289"/>
+      <c r="Q10" s="289"/>
+      <c r="R10" s="289"/>
+      <c r="S10" s="289"/>
+      <c r="T10" s="289"/>
+      <c r="U10" s="289"/>
+      <c r="V10" s="289"/>
+      <c r="W10" s="289"/>
+      <c r="X10" s="289"/>
+      <c r="Y10" s="289"/>
+      <c r="Z10" s="289"/>
+      <c r="AA10" s="289"/>
+      <c r="AB10" s="289"/>
       <c r="AC10" s="64"/>
       <c r="AD10" s="67"/>
       <c r="AE10" s="67"/>
@@ -4672,22 +4678,22 @@
       <c r="AH10" s="70" t="s">
         <v>100</v>
       </c>
-      <c r="AI10" s="293" t="s">
+      <c r="AI10" s="295" t="s">
         <v>3</v>
       </c>
-      <c r="AJ10" s="294"/>
-      <c r="AK10" s="296">
-        <v>94401876</v>
-      </c>
-      <c r="AL10" s="296"/>
-      <c r="AM10" s="296"/>
-      <c r="AN10" s="296"/>
-      <c r="AO10" s="296"/>
-      <c r="AP10" s="296"/>
-      <c r="AQ10" s="296"/>
-      <c r="AR10" s="296"/>
-      <c r="AS10" s="296"/>
-      <c r="AT10" s="297"/>
+      <c r="AJ10" s="296"/>
+      <c r="AK10" s="297">
+        <v>94401877</v>
+      </c>
+      <c r="AL10" s="297"/>
+      <c r="AM10" s="297"/>
+      <c r="AN10" s="297"/>
+      <c r="AO10" s="297"/>
+      <c r="AP10" s="297"/>
+      <c r="AQ10" s="297"/>
+      <c r="AR10" s="297"/>
+      <c r="AS10" s="297"/>
+      <c r="AT10" s="298"/>
       <c r="AU10" s="62"/>
     </row>
     <row r="11" spans="1:47" s="63" customFormat="1" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -4790,55 +4796,55 @@
     </row>
     <row r="13" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="59"/>
-      <c r="B13" s="290" t="s">
+      <c r="B13" s="291" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="290"/>
-      <c r="D13" s="290"/>
-      <c r="E13" s="290"/>
-      <c r="F13" s="290"/>
-      <c r="G13" s="290"/>
-      <c r="H13" s="290"/>
-      <c r="I13" s="298" t="s">
-        <v>105</v>
-      </c>
-      <c r="J13" s="299"/>
-      <c r="K13" s="299"/>
-      <c r="L13" s="299"/>
-      <c r="M13" s="299"/>
-      <c r="N13" s="299"/>
-      <c r="O13" s="299"/>
-      <c r="P13" s="299"/>
-      <c r="Q13" s="299"/>
-      <c r="R13" s="299"/>
-      <c r="S13" s="299"/>
-      <c r="T13" s="299"/>
-      <c r="U13" s="299"/>
-      <c r="V13" s="299"/>
-      <c r="W13" s="299"/>
-      <c r="X13" s="299"/>
-      <c r="Y13" s="299"/>
-      <c r="Z13" s="299"/>
-      <c r="AA13" s="299"/>
-      <c r="AB13" s="299"/>
-      <c r="AC13" s="299"/>
-      <c r="AD13" s="299"/>
-      <c r="AE13" s="299"/>
-      <c r="AF13" s="299"/>
-      <c r="AG13" s="299"/>
-      <c r="AH13" s="299"/>
-      <c r="AI13" s="299"/>
-      <c r="AJ13" s="299"/>
-      <c r="AK13" s="299"/>
-      <c r="AL13" s="299"/>
-      <c r="AM13" s="299"/>
-      <c r="AN13" s="299"/>
-      <c r="AO13" s="299"/>
-      <c r="AP13" s="299"/>
-      <c r="AQ13" s="299"/>
-      <c r="AR13" s="299"/>
-      <c r="AS13" s="299"/>
-      <c r="AT13" s="300"/>
+      <c r="C13" s="291"/>
+      <c r="D13" s="291"/>
+      <c r="E13" s="291"/>
+      <c r="F13" s="291"/>
+      <c r="G13" s="291"/>
+      <c r="H13" s="291"/>
+      <c r="I13" s="299" t="s">
+        <v>103</v>
+      </c>
+      <c r="J13" s="300"/>
+      <c r="K13" s="300"/>
+      <c r="L13" s="300"/>
+      <c r="M13" s="300"/>
+      <c r="N13" s="300"/>
+      <c r="O13" s="300"/>
+      <c r="P13" s="300"/>
+      <c r="Q13" s="300"/>
+      <c r="R13" s="300"/>
+      <c r="S13" s="300"/>
+      <c r="T13" s="300"/>
+      <c r="U13" s="300"/>
+      <c r="V13" s="300"/>
+      <c r="W13" s="300"/>
+      <c r="X13" s="300"/>
+      <c r="Y13" s="300"/>
+      <c r="Z13" s="300"/>
+      <c r="AA13" s="300"/>
+      <c r="AB13" s="300"/>
+      <c r="AC13" s="300"/>
+      <c r="AD13" s="300"/>
+      <c r="AE13" s="300"/>
+      <c r="AF13" s="300"/>
+      <c r="AG13" s="300"/>
+      <c r="AH13" s="300"/>
+      <c r="AI13" s="300"/>
+      <c r="AJ13" s="300"/>
+      <c r="AK13" s="300"/>
+      <c r="AL13" s="300"/>
+      <c r="AM13" s="300"/>
+      <c r="AN13" s="300"/>
+      <c r="AO13" s="300"/>
+      <c r="AP13" s="300"/>
+      <c r="AQ13" s="300"/>
+      <c r="AR13" s="300"/>
+      <c r="AS13" s="300"/>
+      <c r="AT13" s="301"/>
       <c r="AU13" s="62"/>
     </row>
     <row r="14" spans="1:47" s="63" customFormat="1" ht="25" customHeight="1" x14ac:dyDescent="0.35">
@@ -4850,44 +4856,44 @@
       <c r="F14" s="60"/>
       <c r="G14" s="60"/>
       <c r="H14" s="60"/>
-      <c r="I14" s="301"/>
-      <c r="J14" s="302"/>
-      <c r="K14" s="302"/>
-      <c r="L14" s="302"/>
-      <c r="M14" s="302"/>
-      <c r="N14" s="302"/>
-      <c r="O14" s="302"/>
-      <c r="P14" s="302"/>
-      <c r="Q14" s="302"/>
-      <c r="R14" s="302"/>
-      <c r="S14" s="302"/>
-      <c r="T14" s="302"/>
-      <c r="U14" s="302"/>
-      <c r="V14" s="302"/>
-      <c r="W14" s="302"/>
-      <c r="X14" s="302"/>
-      <c r="Y14" s="302"/>
-      <c r="Z14" s="302"/>
-      <c r="AA14" s="302"/>
-      <c r="AB14" s="302"/>
-      <c r="AC14" s="302"/>
-      <c r="AD14" s="302"/>
-      <c r="AE14" s="302"/>
-      <c r="AF14" s="302"/>
-      <c r="AG14" s="302"/>
-      <c r="AH14" s="302"/>
-      <c r="AI14" s="302"/>
-      <c r="AJ14" s="302"/>
-      <c r="AK14" s="302"/>
-      <c r="AL14" s="302"/>
-      <c r="AM14" s="302"/>
-      <c r="AN14" s="302"/>
-      <c r="AO14" s="302"/>
-      <c r="AP14" s="302"/>
-      <c r="AQ14" s="302"/>
-      <c r="AR14" s="302"/>
-      <c r="AS14" s="302"/>
-      <c r="AT14" s="303"/>
+      <c r="I14" s="302"/>
+      <c r="J14" s="303"/>
+      <c r="K14" s="303"/>
+      <c r="L14" s="303"/>
+      <c r="M14" s="303"/>
+      <c r="N14" s="303"/>
+      <c r="O14" s="303"/>
+      <c r="P14" s="303"/>
+      <c r="Q14" s="303"/>
+      <c r="R14" s="303"/>
+      <c r="S14" s="303"/>
+      <c r="T14" s="303"/>
+      <c r="U14" s="303"/>
+      <c r="V14" s="303"/>
+      <c r="W14" s="303"/>
+      <c r="X14" s="303"/>
+      <c r="Y14" s="303"/>
+      <c r="Z14" s="303"/>
+      <c r="AA14" s="303"/>
+      <c r="AB14" s="303"/>
+      <c r="AC14" s="303"/>
+      <c r="AD14" s="303"/>
+      <c r="AE14" s="303"/>
+      <c r="AF14" s="303"/>
+      <c r="AG14" s="303"/>
+      <c r="AH14" s="303"/>
+      <c r="AI14" s="303"/>
+      <c r="AJ14" s="303"/>
+      <c r="AK14" s="303"/>
+      <c r="AL14" s="303"/>
+      <c r="AM14" s="303"/>
+      <c r="AN14" s="303"/>
+      <c r="AO14" s="303"/>
+      <c r="AP14" s="303"/>
+      <c r="AQ14" s="303"/>
+      <c r="AR14" s="303"/>
+      <c r="AS14" s="303"/>
+      <c r="AT14" s="304"/>
       <c r="AU14" s="62"/>
     </row>
     <row r="15" spans="1:47" s="63" customFormat="1" ht="32.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -4899,44 +4905,44 @@
       <c r="F15" s="60"/>
       <c r="G15" s="60"/>
       <c r="H15" s="60"/>
-      <c r="I15" s="304"/>
-      <c r="J15" s="305"/>
-      <c r="K15" s="305"/>
-      <c r="L15" s="305"/>
-      <c r="M15" s="305"/>
-      <c r="N15" s="305"/>
-      <c r="O15" s="305"/>
-      <c r="P15" s="305"/>
-      <c r="Q15" s="305"/>
-      <c r="R15" s="305"/>
-      <c r="S15" s="305"/>
-      <c r="T15" s="305"/>
-      <c r="U15" s="305"/>
-      <c r="V15" s="305"/>
-      <c r="W15" s="305"/>
-      <c r="X15" s="305"/>
-      <c r="Y15" s="305"/>
-      <c r="Z15" s="305"/>
-      <c r="AA15" s="305"/>
-      <c r="AB15" s="305"/>
-      <c r="AC15" s="305"/>
-      <c r="AD15" s="305"/>
-      <c r="AE15" s="305"/>
-      <c r="AF15" s="305"/>
-      <c r="AG15" s="305"/>
-      <c r="AH15" s="305"/>
-      <c r="AI15" s="305"/>
-      <c r="AJ15" s="305"/>
-      <c r="AK15" s="305"/>
-      <c r="AL15" s="305"/>
-      <c r="AM15" s="305"/>
-      <c r="AN15" s="305"/>
-      <c r="AO15" s="305"/>
-      <c r="AP15" s="305"/>
-      <c r="AQ15" s="305"/>
-      <c r="AR15" s="305"/>
-      <c r="AS15" s="305"/>
-      <c r="AT15" s="306"/>
+      <c r="I15" s="305"/>
+      <c r="J15" s="306"/>
+      <c r="K15" s="306"/>
+      <c r="L15" s="306"/>
+      <c r="M15" s="306"/>
+      <c r="N15" s="306"/>
+      <c r="O15" s="306"/>
+      <c r="P15" s="306"/>
+      <c r="Q15" s="306"/>
+      <c r="R15" s="306"/>
+      <c r="S15" s="306"/>
+      <c r="T15" s="306"/>
+      <c r="U15" s="306"/>
+      <c r="V15" s="306"/>
+      <c r="W15" s="306"/>
+      <c r="X15" s="306"/>
+      <c r="Y15" s="306"/>
+      <c r="Z15" s="306"/>
+      <c r="AA15" s="306"/>
+      <c r="AB15" s="306"/>
+      <c r="AC15" s="306"/>
+      <c r="AD15" s="306"/>
+      <c r="AE15" s="306"/>
+      <c r="AF15" s="306"/>
+      <c r="AG15" s="306"/>
+      <c r="AH15" s="306"/>
+      <c r="AI15" s="306"/>
+      <c r="AJ15" s="306"/>
+      <c r="AK15" s="306"/>
+      <c r="AL15" s="306"/>
+      <c r="AM15" s="306"/>
+      <c r="AN15" s="306"/>
+      <c r="AO15" s="306"/>
+      <c r="AP15" s="306"/>
+      <c r="AQ15" s="306"/>
+      <c r="AR15" s="306"/>
+      <c r="AS15" s="306"/>
+      <c r="AT15" s="307"/>
       <c r="AU15" s="62"/>
     </row>
     <row r="16" spans="1:47" s="63" customFormat="1" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -4990,59 +4996,59 @@
     </row>
     <row r="17" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="59"/>
-      <c r="B17" s="290" t="s">
+      <c r="B17" s="291" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="290"/>
-      <c r="D17" s="290"/>
-      <c r="E17" s="290"/>
-      <c r="F17" s="290"/>
-      <c r="G17" s="290"/>
-      <c r="H17" s="290"/>
-      <c r="I17" s="290"/>
-      <c r="J17" s="290"/>
-      <c r="K17" s="290"/>
-      <c r="L17" s="290"/>
-      <c r="M17" s="290" t="s">
+      <c r="C17" s="291"/>
+      <c r="D17" s="291"/>
+      <c r="E17" s="291"/>
+      <c r="F17" s="291"/>
+      <c r="G17" s="291"/>
+      <c r="H17" s="291"/>
+      <c r="I17" s="291"/>
+      <c r="J17" s="291"/>
+      <c r="K17" s="291"/>
+      <c r="L17" s="291"/>
+      <c r="M17" s="291" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="290"/>
-      <c r="O17" s="290"/>
-      <c r="P17" s="290"/>
-      <c r="Q17" s="290"/>
-      <c r="R17" s="334"/>
-      <c r="S17" s="339">
+      <c r="N17" s="291"/>
+      <c r="O17" s="291"/>
+      <c r="P17" s="291"/>
+      <c r="Q17" s="291"/>
+      <c r="R17" s="335"/>
+      <c r="S17" s="340">
         <v>28</v>
       </c>
-      <c r="T17" s="340"/>
-      <c r="U17" s="331">
+      <c r="T17" s="341"/>
+      <c r="U17" s="332">
         <v>4</v>
       </c>
-      <c r="V17" s="332"/>
-      <c r="W17" s="331">
+      <c r="V17" s="333"/>
+      <c r="W17" s="332">
         <v>2025</v>
       </c>
-      <c r="X17" s="333"/>
+      <c r="X17" s="334"/>
       <c r="Y17" s="61"/>
-      <c r="Z17" s="290" t="s">
+      <c r="Z17" s="291" t="s">
         <v>46</v>
       </c>
-      <c r="AA17" s="290"/>
-      <c r="AB17" s="290"/>
-      <c r="AC17" s="290"/>
-      <c r="AD17" s="334"/>
-      <c r="AE17" s="339">
+      <c r="AA17" s="291"/>
+      <c r="AB17" s="291"/>
+      <c r="AC17" s="291"/>
+      <c r="AD17" s="335"/>
+      <c r="AE17" s="340">
         <v>5</v>
       </c>
-      <c r="AF17" s="340"/>
-      <c r="AG17" s="331">
+      <c r="AF17" s="341"/>
+      <c r="AG17" s="332">
         <v>5</v>
       </c>
-      <c r="AH17" s="332"/>
-      <c r="AI17" s="331">
+      <c r="AH17" s="333"/>
+      <c r="AI17" s="332">
         <v>2028</v>
       </c>
-      <c r="AJ17" s="333"/>
+      <c r="AJ17" s="334"/>
       <c r="AK17" s="61"/>
       <c r="AL17" s="61"/>
       <c r="AM17" s="61"/>
@@ -5306,86 +5312,86 @@
     </row>
     <row r="23" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="59"/>
-      <c r="B23" s="344" t="s">
+      <c r="B23" s="345" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="240"/>
-      <c r="D23" s="240"/>
-      <c r="E23" s="240"/>
-      <c r="F23" s="240"/>
-      <c r="G23" s="241"/>
-      <c r="H23" s="239" t="s">
+      <c r="C23" s="241"/>
+      <c r="D23" s="241"/>
+      <c r="E23" s="241"/>
+      <c r="F23" s="241"/>
+      <c r="G23" s="242"/>
+      <c r="H23" s="240" t="s">
         <v>19</v>
       </c>
-      <c r="I23" s="240"/>
-      <c r="J23" s="240"/>
-      <c r="K23" s="240"/>
-      <c r="L23" s="240"/>
-      <c r="M23" s="240"/>
-      <c r="N23" s="240"/>
-      <c r="O23" s="240"/>
-      <c r="P23" s="240"/>
-      <c r="Q23" s="240"/>
-      <c r="R23" s="240"/>
-      <c r="S23" s="240"/>
-      <c r="T23" s="240"/>
-      <c r="U23" s="240"/>
-      <c r="V23" s="241"/>
-      <c r="W23" s="239" t="s">
+      <c r="I23" s="241"/>
+      <c r="J23" s="241"/>
+      <c r="K23" s="241"/>
+      <c r="L23" s="241"/>
+      <c r="M23" s="241"/>
+      <c r="N23" s="241"/>
+      <c r="O23" s="241"/>
+      <c r="P23" s="241"/>
+      <c r="Q23" s="241"/>
+      <c r="R23" s="241"/>
+      <c r="S23" s="241"/>
+      <c r="T23" s="241"/>
+      <c r="U23" s="241"/>
+      <c r="V23" s="242"/>
+      <c r="W23" s="240" t="s">
         <v>24</v>
       </c>
-      <c r="X23" s="240"/>
-      <c r="Y23" s="240"/>
-      <c r="Z23" s="240"/>
-      <c r="AA23" s="240"/>
-      <c r="AB23" s="241"/>
-      <c r="AC23" s="239" t="s">
+      <c r="X23" s="241"/>
+      <c r="Y23" s="241"/>
+      <c r="Z23" s="241"/>
+      <c r="AA23" s="241"/>
+      <c r="AB23" s="242"/>
+      <c r="AC23" s="240" t="s">
         <v>47</v>
       </c>
-      <c r="AD23" s="240"/>
-      <c r="AE23" s="240"/>
-      <c r="AF23" s="240"/>
-      <c r="AG23" s="241"/>
-      <c r="AH23" s="239" t="s">
+      <c r="AD23" s="241"/>
+      <c r="AE23" s="241"/>
+      <c r="AF23" s="241"/>
+      <c r="AG23" s="242"/>
+      <c r="AH23" s="240" t="s">
         <v>27</v>
       </c>
-      <c r="AI23" s="240"/>
-      <c r="AJ23" s="240"/>
-      <c r="AK23" s="240"/>
-      <c r="AL23" s="240"/>
-      <c r="AM23" s="328"/>
-      <c r="AN23" s="344" t="s">
+      <c r="AI23" s="241"/>
+      <c r="AJ23" s="241"/>
+      <c r="AK23" s="241"/>
+      <c r="AL23" s="241"/>
+      <c r="AM23" s="329"/>
+      <c r="AN23" s="345" t="s">
         <v>11</v>
       </c>
-      <c r="AO23" s="240"/>
-      <c r="AP23" s="240"/>
-      <c r="AQ23" s="240"/>
-      <c r="AR23" s="240"/>
-      <c r="AS23" s="240"/>
-      <c r="AT23" s="328"/>
+      <c r="AO23" s="241"/>
+      <c r="AP23" s="241"/>
+      <c r="AQ23" s="241"/>
+      <c r="AR23" s="241"/>
+      <c r="AS23" s="241"/>
+      <c r="AT23" s="329"/>
       <c r="AU23" s="62"/>
     </row>
     <row r="24" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="59"/>
-      <c r="B24" s="345">
+      <c r="B24" s="346">
         <v>45957</v>
       </c>
-      <c r="C24" s="315"/>
-      <c r="D24" s="315"/>
-      <c r="E24" s="315"/>
-      <c r="F24" s="315"/>
-      <c r="G24" s="317"/>
-      <c r="H24" s="314" t="s">
-        <v>107</v>
-      </c>
-      <c r="I24" s="315"/>
-      <c r="J24" s="315"/>
-      <c r="K24" s="315"/>
-      <c r="L24" s="315"/>
-      <c r="M24" s="315"/>
-      <c r="N24" s="315"/>
-      <c r="O24" s="315"/>
-      <c r="P24" s="315"/>
+      <c r="C24" s="316"/>
+      <c r="D24" s="316"/>
+      <c r="E24" s="316"/>
+      <c r="F24" s="316"/>
+      <c r="G24" s="318"/>
+      <c r="H24" s="315" t="s">
+        <v>105</v>
+      </c>
+      <c r="I24" s="316"/>
+      <c r="J24" s="316"/>
+      <c r="K24" s="316"/>
+      <c r="L24" s="316"/>
+      <c r="M24" s="316"/>
+      <c r="N24" s="316"/>
+      <c r="O24" s="316"/>
+      <c r="P24" s="316"/>
       <c r="Q24" s="74"/>
       <c r="R24" s="74"/>
       <c r="S24" s="74"/>
@@ -5394,14 +5400,14 @@
         <v>42</v>
       </c>
       <c r="V24" s="76"/>
-      <c r="W24" s="316">
+      <c r="W24" s="317">
         <v>45961</v>
       </c>
-      <c r="X24" s="315"/>
-      <c r="Y24" s="315"/>
-      <c r="Z24" s="315"/>
-      <c r="AA24" s="315"/>
-      <c r="AB24" s="317"/>
+      <c r="X24" s="316"/>
+      <c r="Y24" s="316"/>
+      <c r="Z24" s="316"/>
+      <c r="AA24" s="316"/>
+      <c r="AB24" s="318"/>
       <c r="AC24" s="77" t="s">
         <v>28</v>
       </c>
@@ -5413,23 +5419,23 @@
         <v>21</v>
       </c>
       <c r="AG24" s="78"/>
-      <c r="AH24" s="316">
+      <c r="AH24" s="317">
         <v>46387</v>
       </c>
-      <c r="AI24" s="315"/>
-      <c r="AJ24" s="315"/>
-      <c r="AK24" s="315"/>
-      <c r="AL24" s="315"/>
-      <c r="AM24" s="318"/>
-      <c r="AN24" s="311">
+      <c r="AI24" s="316"/>
+      <c r="AJ24" s="316"/>
+      <c r="AK24" s="316"/>
+      <c r="AL24" s="316"/>
+      <c r="AM24" s="319"/>
+      <c r="AN24" s="312">
         <v>386128219</v>
       </c>
-      <c r="AO24" s="312"/>
-      <c r="AP24" s="312"/>
-      <c r="AQ24" s="312"/>
-      <c r="AR24" s="312"/>
-      <c r="AS24" s="312"/>
-      <c r="AT24" s="313"/>
+      <c r="AO24" s="313"/>
+      <c r="AP24" s="313"/>
+      <c r="AQ24" s="313"/>
+      <c r="AR24" s="313"/>
+      <c r="AS24" s="313"/>
+      <c r="AT24" s="314"/>
       <c r="AU24" s="62"/>
     </row>
     <row r="25" spans="1:47" ht="35" customHeight="1" x14ac:dyDescent="0.35">
@@ -5483,53 +5489,53 @@
     </row>
     <row r="26" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="59"/>
-      <c r="B26" s="253" t="s">
+      <c r="B26" s="254" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="253"/>
-      <c r="D26" s="253"/>
-      <c r="E26" s="253"/>
-      <c r="F26" s="253"/>
-      <c r="G26" s="253"/>
-      <c r="H26" s="253"/>
-      <c r="I26" s="253"/>
-      <c r="J26" s="253"/>
-      <c r="K26" s="253"/>
-      <c r="L26" s="253"/>
-      <c r="M26" s="253"/>
-      <c r="N26" s="253"/>
-      <c r="O26" s="253"/>
-      <c r="P26" s="253"/>
-      <c r="Q26" s="253"/>
-      <c r="R26" s="253"/>
-      <c r="S26" s="253"/>
-      <c r="T26" s="253"/>
-      <c r="U26" s="253"/>
-      <c r="V26" s="253"/>
-      <c r="W26" s="253"/>
-      <c r="X26" s="253"/>
-      <c r="Y26" s="253"/>
-      <c r="Z26" s="253"/>
-      <c r="AA26" s="253"/>
-      <c r="AB26" s="253"/>
-      <c r="AC26" s="253"/>
-      <c r="AD26" s="253"/>
-      <c r="AE26" s="253"/>
-      <c r="AF26" s="253"/>
-      <c r="AG26" s="253"/>
-      <c r="AH26" s="253"/>
-      <c r="AI26" s="253"/>
-      <c r="AJ26" s="253"/>
-      <c r="AK26" s="253"/>
-      <c r="AL26" s="253"/>
-      <c r="AM26" s="253"/>
-      <c r="AN26" s="253"/>
-      <c r="AO26" s="253"/>
-      <c r="AP26" s="253"/>
-      <c r="AQ26" s="253"/>
-      <c r="AR26" s="253"/>
-      <c r="AS26" s="253"/>
-      <c r="AT26" s="253"/>
+      <c r="C26" s="254"/>
+      <c r="D26" s="254"/>
+      <c r="E26" s="254"/>
+      <c r="F26" s="254"/>
+      <c r="G26" s="254"/>
+      <c r="H26" s="254"/>
+      <c r="I26" s="254"/>
+      <c r="J26" s="254"/>
+      <c r="K26" s="254"/>
+      <c r="L26" s="254"/>
+      <c r="M26" s="254"/>
+      <c r="N26" s="254"/>
+      <c r="O26" s="254"/>
+      <c r="P26" s="254"/>
+      <c r="Q26" s="254"/>
+      <c r="R26" s="254"/>
+      <c r="S26" s="254"/>
+      <c r="T26" s="254"/>
+      <c r="U26" s="254"/>
+      <c r="V26" s="254"/>
+      <c r="W26" s="254"/>
+      <c r="X26" s="254"/>
+      <c r="Y26" s="254"/>
+      <c r="Z26" s="254"/>
+      <c r="AA26" s="254"/>
+      <c r="AB26" s="254"/>
+      <c r="AC26" s="254"/>
+      <c r="AD26" s="254"/>
+      <c r="AE26" s="254"/>
+      <c r="AF26" s="254"/>
+      <c r="AG26" s="254"/>
+      <c r="AH26" s="254"/>
+      <c r="AI26" s="254"/>
+      <c r="AJ26" s="254"/>
+      <c r="AK26" s="254"/>
+      <c r="AL26" s="254"/>
+      <c r="AM26" s="254"/>
+      <c r="AN26" s="254"/>
+      <c r="AO26" s="254"/>
+      <c r="AP26" s="254"/>
+      <c r="AQ26" s="254"/>
+      <c r="AR26" s="254"/>
+      <c r="AS26" s="254"/>
+      <c r="AT26" s="254"/>
       <c r="AU26" s="62"/>
     </row>
     <row r="27" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5537,62 +5543,62 @@
       <c r="B27" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="237" t="s">
+      <c r="C27" s="238" t="s">
         <v>67</v>
       </c>
-      <c r="D27" s="237"/>
-      <c r="E27" s="237"/>
-      <c r="F27" s="237"/>
-      <c r="G27" s="237"/>
-      <c r="H27" s="238"/>
-      <c r="I27" s="324" t="s">
+      <c r="D27" s="238"/>
+      <c r="E27" s="238"/>
+      <c r="F27" s="238"/>
+      <c r="G27" s="238"/>
+      <c r="H27" s="239"/>
+      <c r="I27" s="325" t="s">
         <v>15</v>
       </c>
-      <c r="J27" s="237"/>
-      <c r="K27" s="237"/>
-      <c r="L27" s="237"/>
-      <c r="M27" s="237"/>
-      <c r="N27" s="237"/>
-      <c r="O27" s="237"/>
-      <c r="P27" s="237"/>
-      <c r="Q27" s="237"/>
-      <c r="R27" s="237"/>
-      <c r="S27" s="237"/>
-      <c r="T27" s="237"/>
-      <c r="U27" s="237"/>
-      <c r="V27" s="238"/>
-      <c r="W27" s="324" t="s">
+      <c r="J27" s="238"/>
+      <c r="K27" s="238"/>
+      <c r="L27" s="238"/>
+      <c r="M27" s="238"/>
+      <c r="N27" s="238"/>
+      <c r="O27" s="238"/>
+      <c r="P27" s="238"/>
+      <c r="Q27" s="238"/>
+      <c r="R27" s="238"/>
+      <c r="S27" s="238"/>
+      <c r="T27" s="238"/>
+      <c r="U27" s="238"/>
+      <c r="V27" s="239"/>
+      <c r="W27" s="325" t="s">
         <v>69</v>
       </c>
-      <c r="X27" s="237"/>
-      <c r="Y27" s="237"/>
-      <c r="Z27" s="237"/>
-      <c r="AA27" s="238"/>
-      <c r="AB27" s="324" t="s">
+      <c r="X27" s="238"/>
+      <c r="Y27" s="238"/>
+      <c r="Z27" s="238"/>
+      <c r="AA27" s="239"/>
+      <c r="AB27" s="325" t="s">
         <v>24</v>
       </c>
-      <c r="AC27" s="237"/>
-      <c r="AD27" s="237"/>
-      <c r="AE27" s="237"/>
-      <c r="AF27" s="237"/>
-      <c r="AG27" s="238"/>
-      <c r="AH27" s="324" t="s">
+      <c r="AC27" s="238"/>
+      <c r="AD27" s="238"/>
+      <c r="AE27" s="238"/>
+      <c r="AF27" s="238"/>
+      <c r="AG27" s="239"/>
+      <c r="AH27" s="325" t="s">
         <v>20</v>
       </c>
-      <c r="AI27" s="237"/>
-      <c r="AJ27" s="237"/>
-      <c r="AK27" s="237"/>
-      <c r="AL27" s="237"/>
-      <c r="AM27" s="238"/>
-      <c r="AN27" s="324" t="s">
+      <c r="AI27" s="238"/>
+      <c r="AJ27" s="238"/>
+      <c r="AK27" s="238"/>
+      <c r="AL27" s="238"/>
+      <c r="AM27" s="239"/>
+      <c r="AN27" s="325" t="s">
         <v>68</v>
       </c>
-      <c r="AO27" s="237"/>
-      <c r="AP27" s="237"/>
-      <c r="AQ27" s="237"/>
-      <c r="AR27" s="237"/>
-      <c r="AS27" s="237"/>
-      <c r="AT27" s="325"/>
+      <c r="AO27" s="238"/>
+      <c r="AP27" s="238"/>
+      <c r="AQ27" s="238"/>
+      <c r="AR27" s="238"/>
+      <c r="AS27" s="238"/>
+      <c r="AT27" s="326"/>
       <c r="AU27" s="62"/>
     </row>
     <row r="28" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -5600,68 +5606,68 @@
       <c r="B28" s="80">
         <v>1</v>
       </c>
-      <c r="C28" s="307">
+      <c r="C28" s="308">
         <v>45988</v>
       </c>
-      <c r="D28" s="308"/>
-      <c r="E28" s="308"/>
-      <c r="F28" s="308"/>
-      <c r="G28" s="308"/>
-      <c r="H28" s="308"/>
-      <c r="I28" s="309" t="s">
+      <c r="D28" s="309"/>
+      <c r="E28" s="309"/>
+      <c r="F28" s="309"/>
+      <c r="G28" s="309"/>
+      <c r="H28" s="309"/>
+      <c r="I28" s="310" t="s">
         <v>16</v>
       </c>
-      <c r="J28" s="309"/>
-      <c r="K28" s="310"/>
+      <c r="J28" s="310"/>
+      <c r="K28" s="311"/>
       <c r="L28" s="81"/>
-      <c r="M28" s="326" t="s">
+      <c r="M28" s="327" t="s">
         <v>17</v>
       </c>
-      <c r="N28" s="327"/>
-      <c r="O28" s="327"/>
-      <c r="P28" s="327"/>
+      <c r="N28" s="328"/>
+      <c r="O28" s="328"/>
+      <c r="P28" s="328"/>
       <c r="Q28" s="81"/>
-      <c r="R28" s="329" t="s">
+      <c r="R28" s="330" t="s">
         <v>18</v>
       </c>
-      <c r="S28" s="330"/>
-      <c r="T28" s="330"/>
-      <c r="U28" s="326"/>
+      <c r="S28" s="331"/>
+      <c r="T28" s="331"/>
+      <c r="U28" s="327"/>
       <c r="V28" s="82" t="s">
         <v>100</v>
       </c>
-      <c r="W28" s="335" t="s">
-        <v>148</v>
-      </c>
-      <c r="X28" s="335"/>
-      <c r="Y28" s="335"/>
-      <c r="Z28" s="335"/>
-      <c r="AA28" s="336"/>
-      <c r="AB28" s="337">
+      <c r="W28" s="336" t="s">
+        <v>146</v>
+      </c>
+      <c r="X28" s="336"/>
+      <c r="Y28" s="336"/>
+      <c r="Z28" s="336"/>
+      <c r="AA28" s="337"/>
+      <c r="AB28" s="338">
         <v>46002</v>
       </c>
-      <c r="AC28" s="308"/>
-      <c r="AD28" s="308"/>
-      <c r="AE28" s="308"/>
-      <c r="AF28" s="308"/>
-      <c r="AG28" s="338"/>
-      <c r="AH28" s="321">
+      <c r="AC28" s="309"/>
+      <c r="AD28" s="309"/>
+      <c r="AE28" s="309"/>
+      <c r="AF28" s="309"/>
+      <c r="AG28" s="339"/>
+      <c r="AH28" s="322">
         <v>46367</v>
       </c>
-      <c r="AI28" s="322"/>
-      <c r="AJ28" s="322"/>
-      <c r="AK28" s="322"/>
-      <c r="AL28" s="322"/>
-      <c r="AM28" s="323"/>
-      <c r="AN28" s="346">
+      <c r="AI28" s="323"/>
+      <c r="AJ28" s="323"/>
+      <c r="AK28" s="323"/>
+      <c r="AL28" s="323"/>
+      <c r="AM28" s="324"/>
+      <c r="AN28" s="347">
         <v>389000000</v>
       </c>
-      <c r="AO28" s="346"/>
-      <c r="AP28" s="346"/>
-      <c r="AQ28" s="346"/>
-      <c r="AR28" s="346"/>
-      <c r="AS28" s="346"/>
-      <c r="AT28" s="347"/>
+      <c r="AO28" s="347"/>
+      <c r="AP28" s="347"/>
+      <c r="AQ28" s="347"/>
+      <c r="AR28" s="347"/>
+      <c r="AS28" s="347"/>
+      <c r="AT28" s="348"/>
       <c r="AU28" s="62"/>
     </row>
     <row r="29" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -5677,60 +5683,60 @@
       <c r="F29" s="230"/>
       <c r="G29" s="230"/>
       <c r="H29" s="230"/>
-      <c r="I29" s="256" t="s">
+      <c r="I29" s="257" t="s">
         <v>16</v>
       </c>
-      <c r="J29" s="256"/>
-      <c r="K29" s="257"/>
+      <c r="J29" s="257"/>
+      <c r="K29" s="258"/>
       <c r="L29" s="84"/>
-      <c r="M29" s="260" t="s">
+      <c r="M29" s="261" t="s">
         <v>17</v>
       </c>
-      <c r="N29" s="261"/>
-      <c r="O29" s="261"/>
-      <c r="P29" s="261"/>
+      <c r="N29" s="262"/>
+      <c r="O29" s="262"/>
+      <c r="P29" s="262"/>
       <c r="Q29" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="R29" s="319" t="s">
+      <c r="R29" s="320" t="s">
         <v>18</v>
       </c>
-      <c r="S29" s="320"/>
-      <c r="T29" s="320"/>
-      <c r="U29" s="260"/>
+      <c r="S29" s="321"/>
+      <c r="T29" s="321"/>
+      <c r="U29" s="261"/>
       <c r="V29" s="85"/>
-      <c r="W29" s="270" t="s">
-        <v>149</v>
-      </c>
-      <c r="X29" s="270"/>
-      <c r="Y29" s="270"/>
-      <c r="Z29" s="270"/>
+      <c r="W29" s="271" t="s">
+        <v>147</v>
+      </c>
+      <c r="X29" s="271"/>
+      <c r="Y29" s="271"/>
+      <c r="Z29" s="271"/>
       <c r="AA29" s="218"/>
-      <c r="AB29" s="265">
+      <c r="AB29" s="266">
         <v>46367</v>
       </c>
       <c r="AC29" s="230"/>
       <c r="AD29" s="230"/>
       <c r="AE29" s="230"/>
       <c r="AF29" s="230"/>
-      <c r="AG29" s="266"/>
-      <c r="AH29" s="265">
+      <c r="AG29" s="267"/>
+      <c r="AH29" s="266">
         <v>46733</v>
       </c>
       <c r="AI29" s="230"/>
       <c r="AJ29" s="230"/>
       <c r="AK29" s="230"/>
       <c r="AL29" s="230"/>
-      <c r="AM29" s="266"/>
-      <c r="AN29" s="258">
+      <c r="AM29" s="267"/>
+      <c r="AN29" s="259">
         <v>340999999</v>
       </c>
-      <c r="AO29" s="258"/>
-      <c r="AP29" s="258"/>
-      <c r="AQ29" s="258"/>
-      <c r="AR29" s="258"/>
-      <c r="AS29" s="258"/>
-      <c r="AT29" s="259"/>
+      <c r="AO29" s="259"/>
+      <c r="AP29" s="259"/>
+      <c r="AQ29" s="259"/>
+      <c r="AR29" s="259"/>
+      <c r="AS29" s="259"/>
+      <c r="AT29" s="260"/>
       <c r="AU29" s="62"/>
     </row>
     <row r="30" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -5746,60 +5752,60 @@
       <c r="F30" s="230"/>
       <c r="G30" s="230"/>
       <c r="H30" s="230"/>
-      <c r="I30" s="256" t="s">
+      <c r="I30" s="257" t="s">
         <v>16</v>
       </c>
-      <c r="J30" s="256"/>
-      <c r="K30" s="257"/>
+      <c r="J30" s="257"/>
+      <c r="K30" s="258"/>
       <c r="L30" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="M30" s="260" t="s">
+      <c r="M30" s="261" t="s">
         <v>17</v>
       </c>
-      <c r="N30" s="261"/>
-      <c r="O30" s="261"/>
-      <c r="P30" s="261"/>
+      <c r="N30" s="262"/>
+      <c r="O30" s="262"/>
+      <c r="P30" s="262"/>
       <c r="Q30" s="84"/>
-      <c r="R30" s="319" t="s">
+      <c r="R30" s="320" t="s">
         <v>18</v>
       </c>
-      <c r="S30" s="320"/>
-      <c r="T30" s="320"/>
-      <c r="U30" s="260"/>
+      <c r="S30" s="321"/>
+      <c r="T30" s="321"/>
+      <c r="U30" s="261"/>
       <c r="V30" s="85"/>
-      <c r="W30" s="270" t="s">
-        <v>149</v>
-      </c>
-      <c r="X30" s="270"/>
-      <c r="Y30" s="270"/>
-      <c r="Z30" s="270"/>
+      <c r="W30" s="271" t="s">
+        <v>147</v>
+      </c>
+      <c r="X30" s="271"/>
+      <c r="Y30" s="271"/>
+      <c r="Z30" s="271"/>
       <c r="AA30" s="218"/>
-      <c r="AB30" s="265">
+      <c r="AB30" s="266">
         <v>46338</v>
       </c>
       <c r="AC30" s="230"/>
       <c r="AD30" s="230"/>
       <c r="AE30" s="230"/>
       <c r="AF30" s="230"/>
-      <c r="AG30" s="266"/>
-      <c r="AH30" s="265">
+      <c r="AG30" s="267"/>
+      <c r="AH30" s="266">
         <v>46885</v>
       </c>
       <c r="AI30" s="230"/>
       <c r="AJ30" s="230"/>
       <c r="AK30" s="230"/>
       <c r="AL30" s="230"/>
-      <c r="AM30" s="266"/>
-      <c r="AN30" s="258">
+      <c r="AM30" s="267"/>
+      <c r="AN30" s="259">
         <v>390000544</v>
       </c>
-      <c r="AO30" s="258"/>
-      <c r="AP30" s="258"/>
-      <c r="AQ30" s="258"/>
-      <c r="AR30" s="258"/>
-      <c r="AS30" s="258"/>
-      <c r="AT30" s="259"/>
+      <c r="AO30" s="259"/>
+      <c r="AP30" s="259"/>
+      <c r="AQ30" s="259"/>
+      <c r="AR30" s="259"/>
+      <c r="AS30" s="259"/>
+      <c r="AT30" s="260"/>
       <c r="AU30" s="62"/>
     </row>
     <row r="31" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -5815,60 +5821,60 @@
       <c r="F31" s="230"/>
       <c r="G31" s="230"/>
       <c r="H31" s="230"/>
-      <c r="I31" s="256" t="s">
+      <c r="I31" s="257" t="s">
         <v>16</v>
       </c>
-      <c r="J31" s="256"/>
-      <c r="K31" s="257"/>
+      <c r="J31" s="257"/>
+      <c r="K31" s="258"/>
       <c r="L31" s="84" t="s">
         <v>100</v>
       </c>
-      <c r="M31" s="260" t="s">
+      <c r="M31" s="261" t="s">
         <v>17</v>
       </c>
-      <c r="N31" s="261"/>
-      <c r="O31" s="261"/>
-      <c r="P31" s="261"/>
+      <c r="N31" s="262"/>
+      <c r="O31" s="262"/>
+      <c r="P31" s="262"/>
       <c r="Q31" s="84"/>
-      <c r="R31" s="348" t="s">
+      <c r="R31" s="349" t="s">
         <v>18</v>
       </c>
-      <c r="S31" s="349"/>
-      <c r="T31" s="349"/>
-      <c r="U31" s="350"/>
+      <c r="S31" s="350"/>
+      <c r="T31" s="350"/>
+      <c r="U31" s="351"/>
       <c r="V31" s="85"/>
-      <c r="W31" s="270" t="s">
-        <v>150</v>
-      </c>
-      <c r="X31" s="270"/>
-      <c r="Y31" s="270"/>
-      <c r="Z31" s="270"/>
+      <c r="W31" s="271" t="s">
+        <v>148</v>
+      </c>
+      <c r="X31" s="271"/>
+      <c r="Y31" s="271"/>
+      <c r="Z31" s="271"/>
       <c r="AA31" s="218"/>
-      <c r="AB31" s="265">
+      <c r="AB31" s="266">
         <v>46055</v>
       </c>
       <c r="AC31" s="230"/>
       <c r="AD31" s="230"/>
       <c r="AE31" s="230"/>
       <c r="AF31" s="230"/>
-      <c r="AG31" s="266"/>
-      <c r="AH31" s="265">
+      <c r="AG31" s="267"/>
+      <c r="AH31" s="266">
         <v>46875</v>
       </c>
       <c r="AI31" s="230"/>
       <c r="AJ31" s="230"/>
       <c r="AK31" s="230"/>
       <c r="AL31" s="230"/>
-      <c r="AM31" s="266"/>
-      <c r="AN31" s="258">
+      <c r="AM31" s="267"/>
+      <c r="AN31" s="259">
         <v>400000000</v>
       </c>
-      <c r="AO31" s="258"/>
-      <c r="AP31" s="258"/>
-      <c r="AQ31" s="258"/>
-      <c r="AR31" s="258"/>
-      <c r="AS31" s="258"/>
-      <c r="AT31" s="259"/>
+      <c r="AO31" s="259"/>
+      <c r="AP31" s="259"/>
+      <c r="AQ31" s="259"/>
+      <c r="AR31" s="259"/>
+      <c r="AS31" s="259"/>
+      <c r="AT31" s="260"/>
       <c r="AU31" s="62"/>
     </row>
     <row r="32" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5876,50 +5882,62 @@
       <c r="B32" s="86">
         <v>5</v>
       </c>
-      <c r="C32" s="264"/>
+      <c r="C32" s="265">
+        <v>47538</v>
+      </c>
       <c r="D32" s="108"/>
       <c r="E32" s="108"/>
       <c r="F32" s="108"/>
       <c r="G32" s="108"/>
       <c r="H32" s="108"/>
-      <c r="I32" s="271" t="s">
+      <c r="I32" s="272" t="s">
         <v>16</v>
       </c>
-      <c r="J32" s="271"/>
-      <c r="K32" s="272"/>
+      <c r="J32" s="272"/>
+      <c r="K32" s="273"/>
       <c r="L32" s="87"/>
-      <c r="M32" s="273" t="s">
+      <c r="M32" s="274" t="s">
         <v>17</v>
       </c>
-      <c r="N32" s="274"/>
-      <c r="O32" s="274"/>
-      <c r="P32" s="274"/>
-      <c r="Q32" s="87"/>
-      <c r="R32" s="275" t="s">
+      <c r="N32" s="275"/>
+      <c r="O32" s="275"/>
+      <c r="P32" s="275"/>
+      <c r="Q32" s="87" t="s">
+        <v>100</v>
+      </c>
+      <c r="R32" s="276" t="s">
         <v>18</v>
       </c>
-      <c r="S32" s="276"/>
-      <c r="T32" s="276"/>
-      <c r="U32" s="273"/>
+      <c r="S32" s="277"/>
+      <c r="T32" s="277"/>
+      <c r="U32" s="274"/>
       <c r="V32" s="88"/>
-      <c r="W32" s="105"/>
+      <c r="W32" s="105" t="s">
+        <v>149</v>
+      </c>
       <c r="X32" s="105"/>
       <c r="Y32" s="105"/>
       <c r="Z32" s="105"/>
       <c r="AA32" s="106"/>
-      <c r="AB32" s="341"/>
-      <c r="AC32" s="342"/>
-      <c r="AD32" s="342"/>
-      <c r="AE32" s="342"/>
-      <c r="AF32" s="342"/>
-      <c r="AG32" s="343"/>
-      <c r="AH32" s="110"/>
+      <c r="AB32" s="342">
+        <v>46062</v>
+      </c>
+      <c r="AC32" s="343"/>
+      <c r="AD32" s="343"/>
+      <c r="AE32" s="343"/>
+      <c r="AF32" s="343"/>
+      <c r="AG32" s="344"/>
+      <c r="AH32" s="110">
+        <v>46839</v>
+      </c>
       <c r="AI32" s="111"/>
       <c r="AJ32" s="111"/>
       <c r="AK32" s="111"/>
       <c r="AL32" s="111"/>
       <c r="AM32" s="112"/>
-      <c r="AN32" s="113"/>
+      <c r="AN32" s="113">
+        <v>432555000</v>
+      </c>
       <c r="AO32" s="113"/>
       <c r="AP32" s="113"/>
       <c r="AQ32" s="113"/>
@@ -5933,7 +5951,7 @@
       <c r="B33" s="86">
         <v>6</v>
       </c>
-      <c r="C33" s="264">
+      <c r="C33" s="265">
         <v>46415</v>
       </c>
       <c r="D33" s="108"/>
@@ -5941,25 +5959,25 @@
       <c r="F33" s="108"/>
       <c r="G33" s="108"/>
       <c r="H33" s="108"/>
-      <c r="I33" s="271" t="s">
+      <c r="I33" s="272" t="s">
         <v>16</v>
       </c>
-      <c r="J33" s="271"/>
-      <c r="K33" s="272"/>
+      <c r="J33" s="272"/>
+      <c r="K33" s="273"/>
       <c r="L33" s="87"/>
-      <c r="M33" s="273" t="s">
+      <c r="M33" s="274" t="s">
         <v>17</v>
       </c>
-      <c r="N33" s="274"/>
-      <c r="O33" s="274"/>
-      <c r="P33" s="274"/>
+      <c r="N33" s="275"/>
+      <c r="O33" s="275"/>
+      <c r="P33" s="275"/>
       <c r="Q33" s="87"/>
-      <c r="R33" s="275" t="s">
+      <c r="R33" s="276" t="s">
         <v>18</v>
       </c>
-      <c r="S33" s="276"/>
-      <c r="T33" s="276"/>
-      <c r="U33" s="273"/>
+      <c r="S33" s="277"/>
+      <c r="T33" s="277"/>
+      <c r="U33" s="274"/>
       <c r="V33" s="88" t="s">
         <v>100</v>
       </c>
@@ -6152,38 +6170,38 @@
       <c r="G37" s="1"/>
       <c r="H37" s="1"/>
       <c r="I37" s="1"/>
-      <c r="J37" s="267">
+      <c r="J37" s="268">
         <f>+AN24</f>
         <v>386128219</v>
       </c>
-      <c r="K37" s="267"/>
-      <c r="L37" s="267"/>
-      <c r="M37" s="267"/>
-      <c r="N37" s="267"/>
-      <c r="O37" s="267"/>
-      <c r="P37" s="267"/>
-      <c r="Q37" s="267"/>
-      <c r="R37" s="267"/>
-      <c r="S37" s="267"/>
-      <c r="T37" s="267"/>
-      <c r="U37" s="267"/>
-      <c r="V37" s="267"/>
-      <c r="W37" s="267"/>
-      <c r="X37" s="267"/>
-      <c r="Y37" s="267"/>
-      <c r="Z37" s="267"/>
-      <c r="AA37" s="267"/>
-      <c r="AB37" s="267"/>
-      <c r="AC37" s="267"/>
-      <c r="AD37" s="267"/>
-      <c r="AE37" s="267"/>
-      <c r="AF37" s="267"/>
-      <c r="AG37" s="267"/>
-      <c r="AH37" s="267"/>
-      <c r="AI37" s="267"/>
-      <c r="AJ37" s="267"/>
-      <c r="AK37" s="267"/>
-      <c r="AL37" s="267"/>
+      <c r="K37" s="268"/>
+      <c r="L37" s="268"/>
+      <c r="M37" s="268"/>
+      <c r="N37" s="268"/>
+      <c r="O37" s="268"/>
+      <c r="P37" s="268"/>
+      <c r="Q37" s="268"/>
+      <c r="R37" s="268"/>
+      <c r="S37" s="268"/>
+      <c r="T37" s="268"/>
+      <c r="U37" s="268"/>
+      <c r="V37" s="268"/>
+      <c r="W37" s="268"/>
+      <c r="X37" s="268"/>
+      <c r="Y37" s="268"/>
+      <c r="Z37" s="268"/>
+      <c r="AA37" s="268"/>
+      <c r="AB37" s="268"/>
+      <c r="AC37" s="268"/>
+      <c r="AD37" s="268"/>
+      <c r="AE37" s="268"/>
+      <c r="AF37" s="268"/>
+      <c r="AG37" s="268"/>
+      <c r="AH37" s="268"/>
+      <c r="AI37" s="268"/>
+      <c r="AJ37" s="268"/>
+      <c r="AK37" s="268"/>
+      <c r="AL37" s="268"/>
       <c r="AM37" s="2"/>
       <c r="AN37" s="2"/>
       <c r="AO37" s="2"/>
@@ -6301,60 +6319,60 @@
       <c r="B40" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="268" t="s">
+      <c r="C40" s="269" t="s">
         <v>8</v>
       </c>
-      <c r="D40" s="268"/>
-      <c r="E40" s="268"/>
-      <c r="F40" s="268"/>
-      <c r="G40" s="268"/>
-      <c r="H40" s="269"/>
-      <c r="I40" s="262" t="s">
+      <c r="D40" s="269"/>
+      <c r="E40" s="269"/>
+      <c r="F40" s="269"/>
+      <c r="G40" s="269"/>
+      <c r="H40" s="270"/>
+      <c r="I40" s="263" t="s">
         <v>7</v>
       </c>
-      <c r="J40" s="262"/>
-      <c r="K40" s="262"/>
-      <c r="L40" s="262"/>
-      <c r="M40" s="262"/>
-      <c r="N40" s="262"/>
-      <c r="O40" s="262"/>
-      <c r="P40" s="262"/>
-      <c r="Q40" s="277" t="s">
+      <c r="J40" s="263"/>
+      <c r="K40" s="263"/>
+      <c r="L40" s="263"/>
+      <c r="M40" s="263"/>
+      <c r="N40" s="263"/>
+      <c r="O40" s="263"/>
+      <c r="P40" s="263"/>
+      <c r="Q40" s="278" t="s">
         <v>9</v>
       </c>
-      <c r="R40" s="268"/>
-      <c r="S40" s="268"/>
-      <c r="T40" s="268"/>
-      <c r="U40" s="268"/>
-      <c r="V40" s="268"/>
-      <c r="W40" s="269"/>
-      <c r="X40" s="262" t="s">
+      <c r="R40" s="269"/>
+      <c r="S40" s="269"/>
+      <c r="T40" s="269"/>
+      <c r="U40" s="269"/>
+      <c r="V40" s="269"/>
+      <c r="W40" s="270"/>
+      <c r="X40" s="263" t="s">
         <v>10</v>
       </c>
-      <c r="Y40" s="262"/>
-      <c r="Z40" s="262"/>
-      <c r="AA40" s="262"/>
-      <c r="AB40" s="262"/>
-      <c r="AC40" s="262"/>
-      <c r="AD40" s="262"/>
-      <c r="AE40" s="262"/>
-      <c r="AF40" s="262"/>
-      <c r="AG40" s="262"/>
-      <c r="AH40" s="262"/>
-      <c r="AI40" s="262"/>
-      <c r="AJ40" s="262"/>
-      <c r="AK40" s="262"/>
-      <c r="AL40" s="262"/>
-      <c r="AM40" s="262"/>
-      <c r="AN40" s="262" t="s">
+      <c r="Y40" s="263"/>
+      <c r="Z40" s="263"/>
+      <c r="AA40" s="263"/>
+      <c r="AB40" s="263"/>
+      <c r="AC40" s="263"/>
+      <c r="AD40" s="263"/>
+      <c r="AE40" s="263"/>
+      <c r="AF40" s="263"/>
+      <c r="AG40" s="263"/>
+      <c r="AH40" s="263"/>
+      <c r="AI40" s="263"/>
+      <c r="AJ40" s="263"/>
+      <c r="AK40" s="263"/>
+      <c r="AL40" s="263"/>
+      <c r="AM40" s="263"/>
+      <c r="AN40" s="263" t="s">
         <v>11</v>
       </c>
-      <c r="AO40" s="262"/>
-      <c r="AP40" s="262"/>
-      <c r="AQ40" s="262"/>
-      <c r="AR40" s="262"/>
-      <c r="AS40" s="262"/>
-      <c r="AT40" s="263"/>
+      <c r="AO40" s="263"/>
+      <c r="AP40" s="263"/>
+      <c r="AQ40" s="263"/>
+      <c r="AR40" s="263"/>
+      <c r="AS40" s="263"/>
+      <c r="AT40" s="264"/>
       <c r="AU40" s="14"/>
     </row>
     <row r="41" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -6380,42 +6398,42 @@
       <c r="N41" s="116"/>
       <c r="O41" s="116"/>
       <c r="P41" s="117"/>
-      <c r="Q41" s="244" t="s">
-        <v>108</v>
-      </c>
-      <c r="R41" s="244"/>
-      <c r="S41" s="244"/>
-      <c r="T41" s="244"/>
-      <c r="U41" s="244"/>
-      <c r="V41" s="244"/>
-      <c r="W41" s="244"/>
-      <c r="X41" s="244" t="s">
-        <v>109</v>
-      </c>
-      <c r="Y41" s="244"/>
-      <c r="Z41" s="244"/>
-      <c r="AA41" s="244"/>
-      <c r="AB41" s="244"/>
-      <c r="AC41" s="244"/>
-      <c r="AD41" s="244"/>
-      <c r="AE41" s="244"/>
-      <c r="AF41" s="244"/>
-      <c r="AG41" s="244"/>
-      <c r="AH41" s="244"/>
-      <c r="AI41" s="244"/>
-      <c r="AJ41" s="244"/>
-      <c r="AK41" s="244"/>
-      <c r="AL41" s="244"/>
-      <c r="AM41" s="244"/>
-      <c r="AN41" s="242">
+      <c r="Q41" s="245" t="s">
+        <v>106</v>
+      </c>
+      <c r="R41" s="245"/>
+      <c r="S41" s="245"/>
+      <c r="T41" s="245"/>
+      <c r="U41" s="245"/>
+      <c r="V41" s="245"/>
+      <c r="W41" s="245"/>
+      <c r="X41" s="245" t="s">
+        <v>107</v>
+      </c>
+      <c r="Y41" s="245"/>
+      <c r="Z41" s="245"/>
+      <c r="AA41" s="245"/>
+      <c r="AB41" s="245"/>
+      <c r="AC41" s="245"/>
+      <c r="AD41" s="245"/>
+      <c r="AE41" s="245"/>
+      <c r="AF41" s="245"/>
+      <c r="AG41" s="245"/>
+      <c r="AH41" s="245"/>
+      <c r="AI41" s="245"/>
+      <c r="AJ41" s="245"/>
+      <c r="AK41" s="245"/>
+      <c r="AL41" s="245"/>
+      <c r="AM41" s="245"/>
+      <c r="AN41" s="243">
         <v>86531419</v>
       </c>
-      <c r="AO41" s="242"/>
-      <c r="AP41" s="242"/>
-      <c r="AQ41" s="242"/>
-      <c r="AR41" s="242"/>
-      <c r="AS41" s="242"/>
-      <c r="AT41" s="243"/>
+      <c r="AO41" s="243"/>
+      <c r="AP41" s="243"/>
+      <c r="AQ41" s="243"/>
+      <c r="AR41" s="243"/>
+      <c r="AS41" s="243"/>
+      <c r="AT41" s="244"/>
       <c r="AU41" s="14"/>
     </row>
     <row r="42" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -6438,7 +6456,7 @@
       <c r="O42" s="119"/>
       <c r="P42" s="120"/>
       <c r="Q42" s="179" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="R42" s="179"/>
       <c r="S42" s="179"/>
@@ -6447,7 +6465,7 @@
       <c r="V42" s="179"/>
       <c r="W42" s="179"/>
       <c r="X42" s="179" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="Y42" s="179"/>
       <c r="Z42" s="179"/>
@@ -6480,14 +6498,14 @@
       <c r="B43" s="27">
         <v>3</v>
       </c>
-      <c r="C43" s="371">
+      <c r="C43" s="372">
         <v>46024</v>
       </c>
-      <c r="D43" s="372"/>
-      <c r="E43" s="372"/>
-      <c r="F43" s="372"/>
-      <c r="G43" s="372"/>
-      <c r="H43" s="372"/>
+      <c r="D43" s="373"/>
+      <c r="E43" s="373"/>
+      <c r="F43" s="373"/>
+      <c r="G43" s="373"/>
+      <c r="H43" s="373"/>
       <c r="I43" s="179">
         <v>11263</v>
       </c>
@@ -6499,7 +6517,7 @@
       <c r="O43" s="179"/>
       <c r="P43" s="179"/>
       <c r="Q43" s="179" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="R43" s="179"/>
       <c r="S43" s="179"/>
@@ -6508,7 +6526,7 @@
       <c r="V43" s="179"/>
       <c r="W43" s="179"/>
       <c r="X43" s="179" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Y43" s="179"/>
       <c r="Z43" s="179"/>
@@ -6541,12 +6559,12 @@
       <c r="B44" s="27">
         <v>4</v>
       </c>
-      <c r="C44" s="254"/>
-      <c r="D44" s="255"/>
-      <c r="E44" s="255"/>
-      <c r="F44" s="255"/>
-      <c r="G44" s="255"/>
-      <c r="H44" s="255"/>
+      <c r="C44" s="255"/>
+      <c r="D44" s="256"/>
+      <c r="E44" s="256"/>
+      <c r="F44" s="256"/>
+      <c r="G44" s="256"/>
+      <c r="H44" s="256"/>
       <c r="I44" s="226"/>
       <c r="J44" s="226"/>
       <c r="K44" s="226"/>
@@ -6578,13 +6596,13 @@
       <c r="AK44" s="226"/>
       <c r="AL44" s="226"/>
       <c r="AM44" s="226"/>
-      <c r="AN44" s="366"/>
-      <c r="AO44" s="367"/>
-      <c r="AP44" s="367"/>
-      <c r="AQ44" s="367"/>
-      <c r="AR44" s="367"/>
-      <c r="AS44" s="367"/>
-      <c r="AT44" s="368"/>
+      <c r="AN44" s="367"/>
+      <c r="AO44" s="368"/>
+      <c r="AP44" s="368"/>
+      <c r="AQ44" s="368"/>
+      <c r="AR44" s="368"/>
+      <c r="AS44" s="368"/>
+      <c r="AT44" s="369"/>
       <c r="AU44" s="14"/>
     </row>
     <row r="45" spans="1:47" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6592,12 +6610,12 @@
       <c r="B45" s="28">
         <v>5</v>
       </c>
-      <c r="C45" s="369"/>
-      <c r="D45" s="370"/>
-      <c r="E45" s="370"/>
-      <c r="F45" s="370"/>
-      <c r="G45" s="370"/>
-      <c r="H45" s="370"/>
+      <c r="C45" s="370"/>
+      <c r="D45" s="371"/>
+      <c r="E45" s="371"/>
+      <c r="F45" s="371"/>
+      <c r="G45" s="371"/>
+      <c r="H45" s="371"/>
       <c r="I45" s="227"/>
       <c r="J45" s="227"/>
       <c r="K45" s="227"/>
@@ -6680,16 +6698,16 @@
       <c r="AM46" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="AN46" s="245">
+      <c r="AN46" s="246">
         <f>SUM(AN41:AT45)</f>
         <v>440128219</v>
       </c>
-      <c r="AO46" s="246"/>
-      <c r="AP46" s="246"/>
-      <c r="AQ46" s="246"/>
-      <c r="AR46" s="246"/>
-      <c r="AS46" s="246"/>
-      <c r="AT46" s="247"/>
+      <c r="AO46" s="247"/>
+      <c r="AP46" s="247"/>
+      <c r="AQ46" s="247"/>
+      <c r="AR46" s="247"/>
+      <c r="AS46" s="247"/>
+      <c r="AT46" s="248"/>
       <c r="AU46" s="14"/>
     </row>
     <row r="47" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -6743,53 +6761,53 @@
     </row>
     <row r="48" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="59"/>
-      <c r="B48" s="253" t="s">
+      <c r="B48" s="254" t="s">
         <v>84</v>
       </c>
-      <c r="C48" s="253"/>
-      <c r="D48" s="253"/>
-      <c r="E48" s="253"/>
-      <c r="F48" s="253"/>
-      <c r="G48" s="253"/>
-      <c r="H48" s="253"/>
-      <c r="I48" s="253"/>
-      <c r="J48" s="253"/>
-      <c r="K48" s="253"/>
-      <c r="L48" s="253"/>
-      <c r="M48" s="253"/>
-      <c r="N48" s="253"/>
-      <c r="O48" s="253"/>
-      <c r="P48" s="253"/>
-      <c r="Q48" s="253"/>
-      <c r="R48" s="253"/>
-      <c r="S48" s="253"/>
-      <c r="T48" s="253"/>
-      <c r="U48" s="253"/>
-      <c r="V48" s="253"/>
-      <c r="W48" s="253"/>
-      <c r="X48" s="253"/>
-      <c r="Y48" s="253"/>
-      <c r="Z48" s="253"/>
-      <c r="AA48" s="253"/>
-      <c r="AB48" s="253"/>
-      <c r="AC48" s="253"/>
-      <c r="AD48" s="253"/>
-      <c r="AE48" s="253"/>
-      <c r="AF48" s="253"/>
-      <c r="AG48" s="253"/>
-      <c r="AH48" s="253"/>
-      <c r="AI48" s="253"/>
-      <c r="AJ48" s="253"/>
-      <c r="AK48" s="253"/>
-      <c r="AL48" s="253"/>
-      <c r="AM48" s="253"/>
-      <c r="AN48" s="253"/>
-      <c r="AO48" s="253"/>
-      <c r="AP48" s="253"/>
-      <c r="AQ48" s="253"/>
-      <c r="AR48" s="253"/>
-      <c r="AS48" s="253"/>
-      <c r="AT48" s="253"/>
+      <c r="C48" s="254"/>
+      <c r="D48" s="254"/>
+      <c r="E48" s="254"/>
+      <c r="F48" s="254"/>
+      <c r="G48" s="254"/>
+      <c r="H48" s="254"/>
+      <c r="I48" s="254"/>
+      <c r="J48" s="254"/>
+      <c r="K48" s="254"/>
+      <c r="L48" s="254"/>
+      <c r="M48" s="254"/>
+      <c r="N48" s="254"/>
+      <c r="O48" s="254"/>
+      <c r="P48" s="254"/>
+      <c r="Q48" s="254"/>
+      <c r="R48" s="254"/>
+      <c r="S48" s="254"/>
+      <c r="T48" s="254"/>
+      <c r="U48" s="254"/>
+      <c r="V48" s="254"/>
+      <c r="W48" s="254"/>
+      <c r="X48" s="254"/>
+      <c r="Y48" s="254"/>
+      <c r="Z48" s="254"/>
+      <c r="AA48" s="254"/>
+      <c r="AB48" s="254"/>
+      <c r="AC48" s="254"/>
+      <c r="AD48" s="254"/>
+      <c r="AE48" s="254"/>
+      <c r="AF48" s="254"/>
+      <c r="AG48" s="254"/>
+      <c r="AH48" s="254"/>
+      <c r="AI48" s="254"/>
+      <c r="AJ48" s="254"/>
+      <c r="AK48" s="254"/>
+      <c r="AL48" s="254"/>
+      <c r="AM48" s="254"/>
+      <c r="AN48" s="254"/>
+      <c r="AO48" s="254"/>
+      <c r="AP48" s="254"/>
+      <c r="AQ48" s="254"/>
+      <c r="AR48" s="254"/>
+      <c r="AS48" s="254"/>
+      <c r="AT48" s="254"/>
       <c r="AU48" s="62"/>
     </row>
     <row r="49" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6797,14 +6815,14 @@
       <c r="B49" s="89" t="s">
         <v>21</v>
       </c>
-      <c r="C49" s="237" t="s">
+      <c r="C49" s="238" t="s">
         <v>8</v>
       </c>
-      <c r="D49" s="237"/>
-      <c r="E49" s="237"/>
-      <c r="F49" s="237"/>
-      <c r="G49" s="237"/>
-      <c r="H49" s="238"/>
+      <c r="D49" s="238"/>
+      <c r="E49" s="238"/>
+      <c r="F49" s="238"/>
+      <c r="G49" s="238"/>
+      <c r="H49" s="239"/>
       <c r="I49" s="159" t="s">
         <v>7</v>
       </c>
@@ -6815,15 +6833,15 @@
       <c r="N49" s="159"/>
       <c r="O49" s="159"/>
       <c r="P49" s="159"/>
-      <c r="Q49" s="239" t="s">
+      <c r="Q49" s="240" t="s">
         <v>9</v>
       </c>
-      <c r="R49" s="240"/>
-      <c r="S49" s="240"/>
-      <c r="T49" s="240"/>
-      <c r="U49" s="240"/>
-      <c r="V49" s="240"/>
-      <c r="W49" s="241"/>
+      <c r="R49" s="241"/>
+      <c r="S49" s="241"/>
+      <c r="T49" s="241"/>
+      <c r="U49" s="241"/>
+      <c r="V49" s="241"/>
+      <c r="W49" s="242"/>
       <c r="X49" s="159" t="s">
         <v>10</v>
       </c>
@@ -6858,14 +6876,14 @@
       <c r="B50" s="80">
         <v>1</v>
       </c>
-      <c r="C50" s="351">
+      <c r="C50" s="352">
         <v>45958</v>
       </c>
-      <c r="D50" s="352"/>
-      <c r="E50" s="352"/>
-      <c r="F50" s="352"/>
-      <c r="G50" s="352"/>
-      <c r="H50" s="352"/>
+      <c r="D50" s="353"/>
+      <c r="E50" s="353"/>
+      <c r="F50" s="353"/>
+      <c r="G50" s="353"/>
+      <c r="H50" s="353"/>
       <c r="I50" s="152">
         <v>27254</v>
       </c>
@@ -6876,17 +6894,17 @@
       <c r="N50" s="152"/>
       <c r="O50" s="152"/>
       <c r="P50" s="152"/>
-      <c r="Q50" s="353" t="s">
-        <v>108</v>
-      </c>
-      <c r="R50" s="354"/>
-      <c r="S50" s="354"/>
-      <c r="T50" s="354"/>
-      <c r="U50" s="354"/>
-      <c r="V50" s="354"/>
-      <c r="W50" s="355"/>
+      <c r="Q50" s="354" t="s">
+        <v>106</v>
+      </c>
+      <c r="R50" s="355"/>
+      <c r="S50" s="355"/>
+      <c r="T50" s="355"/>
+      <c r="U50" s="355"/>
+      <c r="V50" s="355"/>
+      <c r="W50" s="356"/>
       <c r="X50" s="152" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Y50" s="152"/>
       <c r="Z50" s="152"/>
@@ -6903,15 +6921,15 @@
       <c r="AK50" s="152"/>
       <c r="AL50" s="152"/>
       <c r="AM50" s="152"/>
-      <c r="AN50" s="248">
+      <c r="AN50" s="249">
         <v>86531419</v>
       </c>
-      <c r="AO50" s="249"/>
-      <c r="AP50" s="249"/>
-      <c r="AQ50" s="249"/>
-      <c r="AR50" s="249"/>
-      <c r="AS50" s="249"/>
-      <c r="AT50" s="250"/>
+      <c r="AO50" s="250"/>
+      <c r="AP50" s="250"/>
+      <c r="AQ50" s="250"/>
+      <c r="AR50" s="250"/>
+      <c r="AS50" s="250"/>
+      <c r="AT50" s="251"/>
       <c r="AU50" s="62"/>
     </row>
     <row r="51" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -6933,32 +6951,32 @@
       <c r="N51" s="219"/>
       <c r="O51" s="219"/>
       <c r="P51" s="219"/>
-      <c r="Q51" s="251" t="s">
-        <v>110</v>
-      </c>
-      <c r="R51" s="252"/>
-      <c r="S51" s="252"/>
-      <c r="T51" s="252"/>
-      <c r="U51" s="252"/>
-      <c r="V51" s="252"/>
+      <c r="Q51" s="252" t="s">
+        <v>108</v>
+      </c>
+      <c r="R51" s="253"/>
+      <c r="S51" s="253"/>
+      <c r="T51" s="253"/>
+      <c r="U51" s="253"/>
+      <c r="V51" s="253"/>
       <c r="W51" s="203"/>
-      <c r="X51" s="251" t="s">
-        <v>111</v>
-      </c>
-      <c r="Y51" s="252"/>
-      <c r="Z51" s="252"/>
-      <c r="AA51" s="252"/>
-      <c r="AB51" s="252"/>
-      <c r="AC51" s="252"/>
-      <c r="AD51" s="252"/>
-      <c r="AE51" s="252"/>
-      <c r="AF51" s="252"/>
-      <c r="AG51" s="252"/>
-      <c r="AH51" s="252"/>
-      <c r="AI51" s="252"/>
-      <c r="AJ51" s="252"/>
-      <c r="AK51" s="252"/>
-      <c r="AL51" s="252"/>
+      <c r="X51" s="252" t="s">
+        <v>109</v>
+      </c>
+      <c r="Y51" s="253"/>
+      <c r="Z51" s="253"/>
+      <c r="AA51" s="253"/>
+      <c r="AB51" s="253"/>
+      <c r="AC51" s="253"/>
+      <c r="AD51" s="253"/>
+      <c r="AE51" s="253"/>
+      <c r="AF51" s="253"/>
+      <c r="AG51" s="253"/>
+      <c r="AH51" s="253"/>
+      <c r="AI51" s="253"/>
+      <c r="AJ51" s="253"/>
+      <c r="AK51" s="253"/>
+      <c r="AL51" s="253"/>
       <c r="AM51" s="203"/>
       <c r="AN51" s="191">
         <v>29596800</v>
@@ -6995,7 +7013,7 @@
       <c r="O52" s="204"/>
       <c r="P52" s="204"/>
       <c r="Q52" s="204" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="R52" s="204"/>
       <c r="S52" s="204"/>
@@ -7004,7 +7022,7 @@
       <c r="V52" s="204"/>
       <c r="W52" s="204"/>
       <c r="X52" s="204" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Y52" s="204"/>
       <c r="Z52" s="204"/>
@@ -7021,15 +7039,15 @@
       <c r="AK52" s="204"/>
       <c r="AL52" s="204"/>
       <c r="AM52" s="204"/>
-      <c r="AN52" s="376">
+      <c r="AN52" s="377">
         <v>324000000</v>
       </c>
-      <c r="AO52" s="376"/>
-      <c r="AP52" s="376"/>
-      <c r="AQ52" s="376"/>
-      <c r="AR52" s="376"/>
-      <c r="AS52" s="376"/>
-      <c r="AT52" s="377"/>
+      <c r="AO52" s="377"/>
+      <c r="AP52" s="377"/>
+      <c r="AQ52" s="377"/>
+      <c r="AR52" s="377"/>
+      <c r="AS52" s="377"/>
+      <c r="AT52" s="378"/>
       <c r="AU52" s="62"/>
     </row>
     <row r="53" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -7051,12 +7069,12 @@
       <c r="N53" s="219"/>
       <c r="O53" s="219"/>
       <c r="P53" s="219"/>
-      <c r="Q53" s="378"/>
-      <c r="R53" s="270"/>
-      <c r="S53" s="270"/>
-      <c r="T53" s="270"/>
-      <c r="U53" s="270"/>
-      <c r="V53" s="270"/>
+      <c r="Q53" s="379"/>
+      <c r="R53" s="271"/>
+      <c r="S53" s="271"/>
+      <c r="T53" s="271"/>
+      <c r="U53" s="271"/>
+      <c r="V53" s="271"/>
       <c r="W53" s="218"/>
       <c r="X53" s="219"/>
       <c r="Y53" s="219"/>
@@ -7088,12 +7106,12 @@
       <c r="B54" s="86">
         <v>5</v>
       </c>
-      <c r="C54" s="379"/>
-      <c r="D54" s="342"/>
-      <c r="E54" s="342"/>
-      <c r="F54" s="342"/>
-      <c r="G54" s="342"/>
-      <c r="H54" s="342"/>
+      <c r="C54" s="380"/>
+      <c r="D54" s="343"/>
+      <c r="E54" s="343"/>
+      <c r="F54" s="343"/>
+      <c r="G54" s="343"/>
+      <c r="H54" s="343"/>
       <c r="I54" s="217"/>
       <c r="J54" s="217"/>
       <c r="K54" s="217"/>
@@ -7102,7 +7120,7 @@
       <c r="N54" s="217"/>
       <c r="O54" s="217"/>
       <c r="P54" s="217"/>
-      <c r="Q54" s="380"/>
+      <c r="Q54" s="381"/>
       <c r="R54" s="105"/>
       <c r="S54" s="105"/>
       <c r="T54" s="105"/>
@@ -7125,13 +7143,13 @@
       <c r="AK54" s="217"/>
       <c r="AL54" s="217"/>
       <c r="AM54" s="217"/>
-      <c r="AN54" s="381"/>
-      <c r="AO54" s="382"/>
-      <c r="AP54" s="382"/>
-      <c r="AQ54" s="382"/>
-      <c r="AR54" s="382"/>
-      <c r="AS54" s="382"/>
-      <c r="AT54" s="383"/>
+      <c r="AN54" s="382"/>
+      <c r="AO54" s="383"/>
+      <c r="AP54" s="383"/>
+      <c r="AQ54" s="383"/>
+      <c r="AR54" s="383"/>
+      <c r="AS54" s="383"/>
+      <c r="AT54" s="384"/>
       <c r="AU54" s="62"/>
     </row>
     <row r="55" spans="1:47" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7176,16 +7194,16 @@
       <c r="AM55" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="AN55" s="373">
+      <c r="AN55" s="374">
         <f>SUM(AN50:AT54)</f>
         <v>440128219</v>
       </c>
-      <c r="AO55" s="374"/>
-      <c r="AP55" s="374"/>
-      <c r="AQ55" s="374"/>
-      <c r="AR55" s="374"/>
-      <c r="AS55" s="374"/>
-      <c r="AT55" s="375"/>
+      <c r="AO55" s="375"/>
+      <c r="AP55" s="375"/>
+      <c r="AQ55" s="375"/>
+      <c r="AR55" s="375"/>
+      <c r="AS55" s="375"/>
+      <c r="AT55" s="376"/>
       <c r="AU55" s="14"/>
     </row>
     <row r="56" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -7339,53 +7357,53 @@
     </row>
     <row r="59" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="59"/>
-      <c r="B59" s="253" t="s">
+      <c r="B59" s="254" t="s">
         <v>95</v>
       </c>
-      <c r="C59" s="253"/>
-      <c r="D59" s="253"/>
-      <c r="E59" s="253"/>
-      <c r="F59" s="253"/>
-      <c r="G59" s="253"/>
-      <c r="H59" s="253"/>
-      <c r="I59" s="253"/>
-      <c r="J59" s="253"/>
-      <c r="K59" s="253"/>
-      <c r="L59" s="253"/>
-      <c r="M59" s="253"/>
-      <c r="N59" s="253"/>
-      <c r="O59" s="253"/>
-      <c r="P59" s="253"/>
-      <c r="Q59" s="253"/>
-      <c r="R59" s="253"/>
-      <c r="S59" s="253"/>
-      <c r="T59" s="253"/>
-      <c r="U59" s="253"/>
-      <c r="V59" s="253"/>
-      <c r="W59" s="253"/>
-      <c r="X59" s="253"/>
-      <c r="Y59" s="253"/>
-      <c r="Z59" s="253"/>
-      <c r="AA59" s="253"/>
-      <c r="AB59" s="253"/>
-      <c r="AC59" s="253"/>
-      <c r="AD59" s="253"/>
-      <c r="AE59" s="253"/>
-      <c r="AF59" s="253"/>
-      <c r="AG59" s="253"/>
-      <c r="AH59" s="253"/>
-      <c r="AI59" s="253"/>
-      <c r="AJ59" s="253"/>
-      <c r="AK59" s="253"/>
-      <c r="AL59" s="253"/>
-      <c r="AM59" s="253"/>
-      <c r="AN59" s="253"/>
-      <c r="AO59" s="253"/>
-      <c r="AP59" s="253"/>
-      <c r="AQ59" s="253"/>
-      <c r="AR59" s="253"/>
-      <c r="AS59" s="253"/>
-      <c r="AT59" s="253"/>
+      <c r="C59" s="254"/>
+      <c r="D59" s="254"/>
+      <c r="E59" s="254"/>
+      <c r="F59" s="254"/>
+      <c r="G59" s="254"/>
+      <c r="H59" s="254"/>
+      <c r="I59" s="254"/>
+      <c r="J59" s="254"/>
+      <c r="K59" s="254"/>
+      <c r="L59" s="254"/>
+      <c r="M59" s="254"/>
+      <c r="N59" s="254"/>
+      <c r="O59" s="254"/>
+      <c r="P59" s="254"/>
+      <c r="Q59" s="254"/>
+      <c r="R59" s="254"/>
+      <c r="S59" s="254"/>
+      <c r="T59" s="254"/>
+      <c r="U59" s="254"/>
+      <c r="V59" s="254"/>
+      <c r="W59" s="254"/>
+      <c r="X59" s="254"/>
+      <c r="Y59" s="254"/>
+      <c r="Z59" s="254"/>
+      <c r="AA59" s="254"/>
+      <c r="AB59" s="254"/>
+      <c r="AC59" s="254"/>
+      <c r="AD59" s="254"/>
+      <c r="AE59" s="254"/>
+      <c r="AF59" s="254"/>
+      <c r="AG59" s="254"/>
+      <c r="AH59" s="254"/>
+      <c r="AI59" s="254"/>
+      <c r="AJ59" s="254"/>
+      <c r="AK59" s="254"/>
+      <c r="AL59" s="254"/>
+      <c r="AM59" s="254"/>
+      <c r="AN59" s="254"/>
+      <c r="AO59" s="254"/>
+      <c r="AP59" s="254"/>
+      <c r="AQ59" s="254"/>
+      <c r="AR59" s="254"/>
+      <c r="AS59" s="254"/>
+      <c r="AT59" s="254"/>
       <c r="AU59" s="62"/>
     </row>
     <row r="60" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7408,24 +7426,24 @@
       <c r="K60" s="159"/>
       <c r="L60" s="159"/>
       <c r="M60" s="159"/>
-      <c r="N60" s="239" t="s">
+      <c r="N60" s="240" t="s">
         <v>71</v>
       </c>
-      <c r="O60" s="240"/>
-      <c r="P60" s="240"/>
-      <c r="Q60" s="240"/>
-      <c r="R60" s="240"/>
-      <c r="S60" s="240"/>
-      <c r="T60" s="240"/>
-      <c r="U60" s="240"/>
-      <c r="V60" s="240"/>
-      <c r="W60" s="240"/>
-      <c r="X60" s="240"/>
-      <c r="Y60" s="240"/>
-      <c r="Z60" s="240"/>
-      <c r="AA60" s="240"/>
-      <c r="AB60" s="240"/>
-      <c r="AC60" s="241"/>
+      <c r="O60" s="241"/>
+      <c r="P60" s="241"/>
+      <c r="Q60" s="241"/>
+      <c r="R60" s="241"/>
+      <c r="S60" s="241"/>
+      <c r="T60" s="241"/>
+      <c r="U60" s="241"/>
+      <c r="V60" s="241"/>
+      <c r="W60" s="241"/>
+      <c r="X60" s="241"/>
+      <c r="Y60" s="241"/>
+      <c r="Z60" s="241"/>
+      <c r="AA60" s="241"/>
+      <c r="AB60" s="241"/>
+      <c r="AC60" s="242"/>
       <c r="AD60" s="159" t="s">
         <v>31</v>
       </c>
@@ -7457,7 +7475,7 @@
         <v>1</v>
       </c>
       <c r="C61" s="228" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D61" s="152"/>
       <c r="E61" s="152"/>
@@ -7465,30 +7483,30 @@
       <c r="G61" s="152"/>
       <c r="H61" s="152"/>
       <c r="I61" s="152" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J61" s="152"/>
       <c r="K61" s="152"/>
       <c r="L61" s="152"/>
       <c r="M61" s="152"/>
-      <c r="N61" s="234" t="s">
-        <v>106</v>
-      </c>
-      <c r="O61" s="235"/>
-      <c r="P61" s="235"/>
-      <c r="Q61" s="235"/>
-      <c r="R61" s="235"/>
-      <c r="S61" s="235"/>
-      <c r="T61" s="235"/>
-      <c r="U61" s="235"/>
-      <c r="V61" s="235"/>
-      <c r="W61" s="235"/>
-      <c r="X61" s="235"/>
-      <c r="Y61" s="235"/>
-      <c r="Z61" s="235"/>
-      <c r="AA61" s="235"/>
-      <c r="AB61" s="235"/>
-      <c r="AC61" s="236"/>
+      <c r="N61" s="235" t="s">
+        <v>104</v>
+      </c>
+      <c r="O61" s="236"/>
+      <c r="P61" s="236"/>
+      <c r="Q61" s="236"/>
+      <c r="R61" s="236"/>
+      <c r="S61" s="236"/>
+      <c r="T61" s="236"/>
+      <c r="U61" s="236"/>
+      <c r="V61" s="236"/>
+      <c r="W61" s="236"/>
+      <c r="X61" s="236"/>
+      <c r="Y61" s="236"/>
+      <c r="Z61" s="236"/>
+      <c r="AA61" s="236"/>
+      <c r="AB61" s="236"/>
+      <c r="AC61" s="237"/>
       <c r="AD61" s="151">
         <v>45957</v>
       </c>
@@ -7503,15 +7521,15 @@
       <c r="AK61" s="151"/>
       <c r="AL61" s="151"/>
       <c r="AM61" s="151"/>
-      <c r="AN61" s="248">
+      <c r="AN61" s="249">
         <v>77225643.799999997</v>
       </c>
-      <c r="AO61" s="249"/>
-      <c r="AP61" s="249"/>
-      <c r="AQ61" s="249"/>
-      <c r="AR61" s="249"/>
-      <c r="AS61" s="249"/>
-      <c r="AT61" s="250"/>
+      <c r="AO61" s="250"/>
+      <c r="AP61" s="250"/>
+      <c r="AQ61" s="250"/>
+      <c r="AR61" s="250"/>
+      <c r="AS61" s="250"/>
+      <c r="AT61" s="251"/>
       <c r="AU61" s="62"/>
     </row>
     <row r="62" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -7531,7 +7549,7 @@
       <c r="L62" s="152"/>
       <c r="M62" s="152"/>
       <c r="N62" s="223" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="O62" s="224"/>
       <c r="P62" s="224"/>
@@ -7548,20 +7566,20 @@
       <c r="AA62" s="224"/>
       <c r="AB62" s="224"/>
       <c r="AC62" s="225"/>
-      <c r="AD62" s="151">
+      <c r="AD62" s="233">
         <v>45957</v>
       </c>
-      <c r="AE62" s="151"/>
-      <c r="AF62" s="151"/>
-      <c r="AG62" s="151"/>
-      <c r="AH62" s="151"/>
-      <c r="AI62" s="233">
+      <c r="AE62" s="233"/>
+      <c r="AF62" s="233"/>
+      <c r="AG62" s="233"/>
+      <c r="AH62" s="233"/>
+      <c r="AI62" s="234">
         <v>46568</v>
       </c>
-      <c r="AJ62" s="233"/>
-      <c r="AK62" s="233"/>
-      <c r="AL62" s="233"/>
-      <c r="AM62" s="233"/>
+      <c r="AJ62" s="234"/>
+      <c r="AK62" s="234"/>
+      <c r="AL62" s="234"/>
+      <c r="AM62" s="234"/>
       <c r="AN62" s="191">
         <v>77225643.799999997</v>
       </c>
@@ -7590,7 +7608,7 @@
       <c r="L63" s="152"/>
       <c r="M63" s="152"/>
       <c r="N63" s="223" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="O63" s="224"/>
       <c r="P63" s="224"/>
@@ -7614,13 +7632,13 @@
       <c r="AF63" s="151"/>
       <c r="AG63" s="151"/>
       <c r="AH63" s="151"/>
-      <c r="AI63" s="233">
+      <c r="AI63" s="234">
         <v>47483</v>
       </c>
-      <c r="AJ63" s="233"/>
-      <c r="AK63" s="233"/>
-      <c r="AL63" s="233"/>
-      <c r="AM63" s="233"/>
+      <c r="AJ63" s="234"/>
+      <c r="AK63" s="234"/>
+      <c r="AL63" s="234"/>
+      <c r="AM63" s="234"/>
       <c r="AN63" s="191">
         <v>38612821.899999999</v>
       </c>
@@ -7638,7 +7656,7 @@
         <v>4</v>
       </c>
       <c r="C64" s="218" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D64" s="219"/>
       <c r="E64" s="219"/>
@@ -7650,8 +7668,8 @@
       <c r="K64" s="219"/>
       <c r="L64" s="219"/>
       <c r="M64" s="219"/>
-      <c r="N64" s="390" t="s">
-        <v>146</v>
+      <c r="N64" s="391" t="s">
+        <v>144</v>
       </c>
       <c r="O64" s="224"/>
       <c r="P64" s="224"/>
@@ -7682,15 +7700,15 @@
       <c r="AK64" s="222"/>
       <c r="AL64" s="222"/>
       <c r="AM64" s="222"/>
-      <c r="AN64" s="359">
+      <c r="AN64" s="360">
         <v>56654212.869999997</v>
       </c>
-      <c r="AO64" s="360"/>
-      <c r="AP64" s="360"/>
-      <c r="AQ64" s="360"/>
-      <c r="AR64" s="360"/>
-      <c r="AS64" s="360"/>
-      <c r="AT64" s="361"/>
+      <c r="AO64" s="361"/>
+      <c r="AP64" s="361"/>
+      <c r="AQ64" s="361"/>
+      <c r="AR64" s="361"/>
+      <c r="AS64" s="361"/>
+      <c r="AT64" s="362"/>
       <c r="AU64" s="62"/>
     </row>
     <row r="65" spans="1:47" s="63" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7709,39 +7727,39 @@
       <c r="K65" s="217"/>
       <c r="L65" s="217"/>
       <c r="M65" s="217"/>
-      <c r="N65" s="356"/>
-      <c r="O65" s="357"/>
-      <c r="P65" s="357"/>
-      <c r="Q65" s="357"/>
-      <c r="R65" s="357"/>
-      <c r="S65" s="357"/>
-      <c r="T65" s="357"/>
-      <c r="U65" s="357"/>
-      <c r="V65" s="357"/>
-      <c r="W65" s="357"/>
-      <c r="X65" s="357"/>
-      <c r="Y65" s="357"/>
-      <c r="Z65" s="357"/>
-      <c r="AA65" s="357"/>
-      <c r="AB65" s="357"/>
-      <c r="AC65" s="358"/>
-      <c r="AD65" s="362"/>
-      <c r="AE65" s="362"/>
-      <c r="AF65" s="362"/>
-      <c r="AG65" s="362"/>
-      <c r="AH65" s="362"/>
-      <c r="AI65" s="362"/>
-      <c r="AJ65" s="362"/>
-      <c r="AK65" s="362"/>
-      <c r="AL65" s="362"/>
-      <c r="AM65" s="362"/>
-      <c r="AN65" s="387"/>
-      <c r="AO65" s="388"/>
-      <c r="AP65" s="388"/>
-      <c r="AQ65" s="388"/>
-      <c r="AR65" s="388"/>
-      <c r="AS65" s="388"/>
-      <c r="AT65" s="389"/>
+      <c r="N65" s="357"/>
+      <c r="O65" s="358"/>
+      <c r="P65" s="358"/>
+      <c r="Q65" s="358"/>
+      <c r="R65" s="358"/>
+      <c r="S65" s="358"/>
+      <c r="T65" s="358"/>
+      <c r="U65" s="358"/>
+      <c r="V65" s="358"/>
+      <c r="W65" s="358"/>
+      <c r="X65" s="358"/>
+      <c r="Y65" s="358"/>
+      <c r="Z65" s="358"/>
+      <c r="AA65" s="358"/>
+      <c r="AB65" s="358"/>
+      <c r="AC65" s="359"/>
+      <c r="AD65" s="363"/>
+      <c r="AE65" s="363"/>
+      <c r="AF65" s="363"/>
+      <c r="AG65" s="363"/>
+      <c r="AH65" s="363"/>
+      <c r="AI65" s="363"/>
+      <c r="AJ65" s="363"/>
+      <c r="AK65" s="363"/>
+      <c r="AL65" s="363"/>
+      <c r="AM65" s="363"/>
+      <c r="AN65" s="388"/>
+      <c r="AO65" s="389"/>
+      <c r="AP65" s="389"/>
+      <c r="AQ65" s="389"/>
+      <c r="AR65" s="389"/>
+      <c r="AS65" s="389"/>
+      <c r="AT65" s="390"/>
       <c r="AU65" s="62"/>
     </row>
     <row r="66" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
@@ -7903,32 +7921,32 @@
       <c r="G69" s="48"/>
       <c r="H69" s="48"/>
       <c r="I69" s="2"/>
-      <c r="J69" s="391"/>
-      <c r="K69" s="391"/>
-      <c r="L69" s="391"/>
-      <c r="M69" s="391"/>
-      <c r="N69" s="391"/>
-      <c r="O69" s="391"/>
-      <c r="P69" s="391"/>
-      <c r="Q69" s="391"/>
-      <c r="R69" s="391"/>
-      <c r="S69" s="391"/>
-      <c r="T69" s="391"/>
-      <c r="U69" s="391"/>
-      <c r="V69" s="391"/>
-      <c r="W69" s="391"/>
-      <c r="X69" s="391"/>
-      <c r="Y69" s="391"/>
-      <c r="Z69" s="391"/>
-      <c r="AA69" s="391"/>
-      <c r="AB69" s="391"/>
-      <c r="AC69" s="391"/>
-      <c r="AD69" s="391"/>
-      <c r="AE69" s="391"/>
-      <c r="AF69" s="391"/>
-      <c r="AG69" s="391"/>
-      <c r="AH69" s="391"/>
-      <c r="AI69" s="391"/>
+      <c r="J69" s="392"/>
+      <c r="K69" s="392"/>
+      <c r="L69" s="392"/>
+      <c r="M69" s="392"/>
+      <c r="N69" s="392"/>
+      <c r="O69" s="392"/>
+      <c r="P69" s="392"/>
+      <c r="Q69" s="392"/>
+      <c r="R69" s="392"/>
+      <c r="S69" s="392"/>
+      <c r="T69" s="392"/>
+      <c r="U69" s="392"/>
+      <c r="V69" s="392"/>
+      <c r="W69" s="392"/>
+      <c r="X69" s="392"/>
+      <c r="Y69" s="392"/>
+      <c r="Z69" s="392"/>
+      <c r="AA69" s="392"/>
+      <c r="AB69" s="392"/>
+      <c r="AC69" s="392"/>
+      <c r="AD69" s="392"/>
+      <c r="AE69" s="392"/>
+      <c r="AF69" s="392"/>
+      <c r="AG69" s="392"/>
+      <c r="AH69" s="392"/>
+      <c r="AI69" s="392"/>
       <c r="AJ69" s="2"/>
       <c r="AK69" s="2"/>
       <c r="AL69" s="2"/>
@@ -8004,7 +8022,7 @@
       <c r="AQ70" s="206"/>
       <c r="AR70" s="206"/>
       <c r="AS70" s="206"/>
-      <c r="AT70" s="384"/>
+      <c r="AT70" s="385"/>
       <c r="AU70" s="14"/>
     </row>
     <row r="71" spans="1:47" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -8043,7 +8061,7 @@
       <c r="AG71" s="216"/>
       <c r="AH71" s="216"/>
       <c r="AI71" s="216"/>
-      <c r="AJ71" s="385"/>
+      <c r="AJ71" s="386"/>
       <c r="AK71" s="208"/>
       <c r="AL71" s="208"/>
       <c r="AM71" s="208"/>
@@ -8053,7 +8071,7 @@
       <c r="AQ71" s="208"/>
       <c r="AR71" s="208"/>
       <c r="AS71" s="208"/>
-      <c r="AT71" s="386"/>
+      <c r="AT71" s="387"/>
       <c r="AU71" s="14"/>
     </row>
     <row r="72" spans="1:47" ht="130" customHeight="1" x14ac:dyDescent="0.35">
@@ -8065,7 +8083,7 @@
       <c r="D72" s="128"/>
       <c r="E72" s="129"/>
       <c r="F72" s="130" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="G72" s="130"/>
       <c r="H72" s="130"/>
@@ -8091,7 +8109,7 @@
       <c r="AB72" s="131"/>
       <c r="AC72" s="131"/>
       <c r="AD72" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE72" s="133"/>
       <c r="AF72" s="134"/>
@@ -8120,7 +8138,7 @@
       <c r="D73" s="128"/>
       <c r="E73" s="129"/>
       <c r="F73" s="130" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="G73" s="130"/>
       <c r="H73" s="130"/>
@@ -8146,7 +8164,7 @@
       <c r="AB73" s="131"/>
       <c r="AC73" s="131"/>
       <c r="AD73" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE73" s="133"/>
       <c r="AF73" s="134"/>
@@ -8175,7 +8193,7 @@
       <c r="D74" s="128"/>
       <c r="E74" s="129"/>
       <c r="F74" s="130" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="G74" s="130"/>
       <c r="H74" s="130"/>
@@ -8193,7 +8211,7 @@
       <c r="T74" s="130"/>
       <c r="U74" s="130"/>
       <c r="V74" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="W74" s="131"/>
       <c r="X74" s="131"/>
@@ -8209,7 +8227,7 @@
       <c r="AH74" s="133"/>
       <c r="AI74" s="134"/>
       <c r="AJ74" s="138" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="AK74" s="139"/>
       <c r="AL74" s="139"/>
@@ -8232,7 +8250,7 @@
       <c r="D75" s="128"/>
       <c r="E75" s="129"/>
       <c r="F75" s="130" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="G75" s="130"/>
       <c r="H75" s="130"/>
@@ -8250,7 +8268,7 @@
       <c r="T75" s="130"/>
       <c r="U75" s="130"/>
       <c r="V75" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="W75" s="131"/>
       <c r="X75" s="131"/>
@@ -8266,7 +8284,7 @@
       <c r="AH75" s="133"/>
       <c r="AI75" s="134"/>
       <c r="AJ75" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK75" s="139"/>
       <c r="AL75" s="139"/>
@@ -8289,7 +8307,7 @@
       <c r="D76" s="128"/>
       <c r="E76" s="129"/>
       <c r="F76" s="130" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G76" s="130"/>
       <c r="H76" s="130"/>
@@ -8315,7 +8333,7 @@
       <c r="AB76" s="131"/>
       <c r="AC76" s="131"/>
       <c r="AD76" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE76" s="133"/>
       <c r="AF76" s="134"/>
@@ -8344,7 +8362,7 @@
       <c r="D77" s="128"/>
       <c r="E77" s="129"/>
       <c r="F77" s="130" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G77" s="130"/>
       <c r="H77" s="130"/>
@@ -8362,7 +8380,7 @@
       <c r="T77" s="130"/>
       <c r="U77" s="130"/>
       <c r="V77" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="W77" s="131"/>
       <c r="X77" s="131"/>
@@ -8378,7 +8396,7 @@
       <c r="AH77" s="133"/>
       <c r="AI77" s="134"/>
       <c r="AJ77" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK77" s="139"/>
       <c r="AL77" s="139"/>
@@ -8401,7 +8419,7 @@
       <c r="D78" s="128"/>
       <c r="E78" s="129"/>
       <c r="F78" s="130" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G78" s="130"/>
       <c r="H78" s="130"/>
@@ -8419,7 +8437,7 @@
       <c r="T78" s="130"/>
       <c r="U78" s="130"/>
       <c r="V78" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="W78" s="131"/>
       <c r="X78" s="131"/>
@@ -8435,7 +8453,7 @@
       <c r="AH78" s="133"/>
       <c r="AI78" s="134"/>
       <c r="AJ78" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK78" s="139"/>
       <c r="AL78" s="139"/>
@@ -8458,7 +8476,7 @@
       <c r="D79" s="128"/>
       <c r="E79" s="129"/>
       <c r="F79" s="130" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="G79" s="130"/>
       <c r="H79" s="130"/>
@@ -8484,7 +8502,7 @@
       <c r="AB79" s="131"/>
       <c r="AC79" s="131"/>
       <c r="AD79" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE79" s="133"/>
       <c r="AF79" s="134"/>
@@ -8513,7 +8531,7 @@
       <c r="D80" s="128"/>
       <c r="E80" s="129"/>
       <c r="F80" s="130" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G80" s="130"/>
       <c r="H80" s="130"/>
@@ -8536,7 +8554,7 @@
       <c r="Y80" s="131"/>
       <c r="Z80" s="131"/>
       <c r="AA80" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB80" s="131"/>
       <c r="AC80" s="131"/>
@@ -8547,7 +8565,7 @@
       <c r="AH80" s="133"/>
       <c r="AI80" s="134"/>
       <c r="AJ80" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK80" s="139"/>
       <c r="AL80" s="139"/>
@@ -8570,7 +8588,7 @@
       <c r="D81" s="128"/>
       <c r="E81" s="129"/>
       <c r="F81" s="130" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G81" s="130"/>
       <c r="H81" s="130"/>
@@ -8593,7 +8611,7 @@
       <c r="Y81" s="131"/>
       <c r="Z81" s="131"/>
       <c r="AA81" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB81" s="131"/>
       <c r="AC81" s="131"/>
@@ -8604,7 +8622,7 @@
       <c r="AH81" s="133"/>
       <c r="AI81" s="134"/>
       <c r="AJ81" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK81" s="139"/>
       <c r="AL81" s="139"/>
@@ -8627,7 +8645,7 @@
       <c r="D82" s="128"/>
       <c r="E82" s="129"/>
       <c r="F82" s="130" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="G82" s="130"/>
       <c r="H82" s="130"/>
@@ -8650,7 +8668,7 @@
       <c r="Y82" s="131"/>
       <c r="Z82" s="131"/>
       <c r="AA82" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AB82" s="131"/>
       <c r="AC82" s="131"/>
@@ -8661,7 +8679,7 @@
       <c r="AH82" s="133"/>
       <c r="AI82" s="134"/>
       <c r="AJ82" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK82" s="139"/>
       <c r="AL82" s="139"/>
@@ -8684,7 +8702,7 @@
       <c r="D83" s="128"/>
       <c r="E83" s="129"/>
       <c r="F83" s="130" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G83" s="130"/>
       <c r="H83" s="130"/>
@@ -8710,7 +8728,7 @@
       <c r="AB83" s="131"/>
       <c r="AC83" s="131"/>
       <c r="AD83" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE83" s="133"/>
       <c r="AF83" s="134"/>
@@ -8739,7 +8757,7 @@
       <c r="D84" s="128"/>
       <c r="E84" s="129"/>
       <c r="F84" s="130" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G84" s="130"/>
       <c r="H84" s="130"/>
@@ -8765,7 +8783,7 @@
       <c r="AB84" s="131"/>
       <c r="AC84" s="131"/>
       <c r="AD84" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE84" s="133"/>
       <c r="AF84" s="134"/>
@@ -8794,7 +8812,7 @@
       <c r="D85" s="128"/>
       <c r="E85" s="129"/>
       <c r="F85" s="130" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="G85" s="130"/>
       <c r="H85" s="130"/>
@@ -8820,7 +8838,7 @@
       <c r="AB85" s="131"/>
       <c r="AC85" s="131"/>
       <c r="AD85" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE85" s="133"/>
       <c r="AF85" s="134"/>
@@ -8849,7 +8867,7 @@
       <c r="D86" s="128"/>
       <c r="E86" s="129"/>
       <c r="F86" s="130" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G86" s="130"/>
       <c r="H86" s="130"/>
@@ -8875,7 +8893,7 @@
       <c r="AB86" s="131"/>
       <c r="AC86" s="131"/>
       <c r="AD86" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE86" s="133"/>
       <c r="AF86" s="134"/>
@@ -8904,7 +8922,7 @@
       <c r="D87" s="128"/>
       <c r="E87" s="129"/>
       <c r="F87" s="130" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="G87" s="130"/>
       <c r="H87" s="130"/>
@@ -8930,7 +8948,7 @@
       <c r="AB87" s="131"/>
       <c r="AC87" s="131"/>
       <c r="AD87" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE87" s="133"/>
       <c r="AF87" s="134"/>
@@ -8959,7 +8977,7 @@
       <c r="D88" s="128"/>
       <c r="E88" s="129"/>
       <c r="F88" s="130" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="G88" s="130"/>
       <c r="H88" s="130"/>
@@ -8977,7 +8995,7 @@
       <c r="T88" s="130"/>
       <c r="U88" s="130"/>
       <c r="V88" s="131" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="W88" s="131"/>
       <c r="X88" s="131"/>
@@ -8993,7 +9011,7 @@
       <c r="AH88" s="133"/>
       <c r="AI88" s="134"/>
       <c r="AJ88" s="138" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="AK88" s="139"/>
       <c r="AL88" s="139"/>
@@ -9016,7 +9034,7 @@
       <c r="D89" s="128"/>
       <c r="E89" s="129"/>
       <c r="F89" s="130" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="G89" s="130"/>
       <c r="H89" s="130"/>
@@ -9042,7 +9060,7 @@
       <c r="AB89" s="131"/>
       <c r="AC89" s="131"/>
       <c r="AD89" s="132" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="AE89" s="133"/>
       <c r="AF89" s="134"/>
@@ -9924,25 +9942,25 @@
       <c r="J107" s="147"/>
       <c r="K107" s="147"/>
       <c r="L107" s="147"/>
-      <c r="M107" s="417" t="s">
+      <c r="M107" s="418" t="s">
         <v>48</v>
       </c>
-      <c r="N107" s="417"/>
-      <c r="O107" s="417"/>
-      <c r="P107" s="417" t="s">
+      <c r="N107" s="418"/>
+      <c r="O107" s="418"/>
+      <c r="P107" s="418" t="s">
         <v>59</v>
       </c>
-      <c r="Q107" s="417"/>
-      <c r="R107" s="417"/>
-      <c r="S107" s="417" t="s">
+      <c r="Q107" s="418"/>
+      <c r="R107" s="418"/>
+      <c r="S107" s="418" t="s">
         <v>50</v>
       </c>
-      <c r="T107" s="417"/>
-      <c r="U107" s="417"/>
-      <c r="V107" s="417" t="s">
+      <c r="T107" s="418"/>
+      <c r="U107" s="418"/>
+      <c r="V107" s="418" t="s">
         <v>60</v>
       </c>
-      <c r="W107" s="417"/>
+      <c r="W107" s="418"/>
       <c r="X107" s="147" t="s">
         <v>51</v>
       </c>
@@ -9985,7 +10003,7 @@
       <c r="F108" s="190"/>
       <c r="G108" s="190"/>
       <c r="H108" s="177" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="I108" s="177"/>
       <c r="J108" s="177"/>
@@ -10011,7 +10029,7 @@
       </c>
       <c r="W108" s="177"/>
       <c r="X108" s="176" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="Y108" s="176"/>
       <c r="Z108" s="176"/>
@@ -10530,7 +10548,7 @@
       <c r="F118" s="151"/>
       <c r="G118" s="151"/>
       <c r="H118" s="152" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I118" s="152"/>
       <c r="J118" s="152"/>
@@ -10556,7 +10574,7 @@
       </c>
       <c r="W118" s="152"/>
       <c r="X118" s="153" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="Y118" s="153"/>
       <c r="Z118" s="153"/>
@@ -11300,20 +11318,20 @@
     </row>
     <row r="135" spans="1:62" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="13"/>
-      <c r="B135" s="416" t="s">
+      <c r="B135" s="417" t="s">
         <v>61</v>
       </c>
-      <c r="C135" s="416"/>
-      <c r="D135" s="416"/>
-      <c r="E135" s="416"/>
-      <c r="F135" s="416"/>
-      <c r="G135" s="416"/>
-      <c r="H135" s="416"/>
-      <c r="I135" s="416"/>
-      <c r="J135" s="416"/>
-      <c r="K135" s="416"/>
+      <c r="C135" s="417"/>
+      <c r="D135" s="417"/>
+      <c r="E135" s="417"/>
+      <c r="F135" s="417"/>
+      <c r="G135" s="417"/>
+      <c r="H135" s="417"/>
+      <c r="I135" s="417"/>
+      <c r="J135" s="417"/>
+      <c r="K135" s="417"/>
       <c r="L135" s="154" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="M135" s="154"/>
       <c r="N135" s="154"/>
@@ -11344,13 +11362,13 @@
       <c r="AK135" s="50"/>
       <c r="AL135" s="50"/>
       <c r="AM135" s="31"/>
-      <c r="AN135" s="404"/>
-      <c r="AO135" s="405"/>
-      <c r="AP135" s="405"/>
-      <c r="AQ135" s="405"/>
-      <c r="AR135" s="405"/>
-      <c r="AS135" s="405"/>
-      <c r="AT135" s="406"/>
+      <c r="AN135" s="405"/>
+      <c r="AO135" s="406"/>
+      <c r="AP135" s="406"/>
+      <c r="AQ135" s="406"/>
+      <c r="AR135" s="406"/>
+      <c r="AS135" s="406"/>
+      <c r="AT135" s="407"/>
       <c r="AU135" s="14"/>
       <c r="AZ135" s="56">
         <f>+AZ134/1.19</f>
@@ -11359,18 +11377,18 @@
     </row>
     <row r="136" spans="1:62" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A136" s="13"/>
-      <c r="B136" s="397" t="s">
+      <c r="B136" s="398" t="s">
         <v>62</v>
       </c>
-      <c r="C136" s="397"/>
-      <c r="D136" s="397"/>
-      <c r="E136" s="397"/>
-      <c r="F136" s="397"/>
-      <c r="G136" s="397"/>
-      <c r="H136" s="397"/>
-      <c r="I136" s="397"/>
-      <c r="J136" s="397"/>
-      <c r="K136" s="397"/>
+      <c r="C136" s="398"/>
+      <c r="D136" s="398"/>
+      <c r="E136" s="398"/>
+      <c r="F136" s="398"/>
+      <c r="G136" s="398"/>
+      <c r="H136" s="398"/>
+      <c r="I136" s="398"/>
+      <c r="J136" s="398"/>
+      <c r="K136" s="398"/>
       <c r="L136" s="155"/>
       <c r="M136" s="155"/>
       <c r="N136" s="155"/>
@@ -11392,10 +11410,10 @@
       <c r="AB136" s="55"/>
       <c r="AC136" s="55"/>
       <c r="AD136" s="31"/>
-      <c r="AE136" s="399">
+      <c r="AE136" s="400">
         <v>44275</v>
       </c>
-      <c r="AF136" s="400"/>
+      <c r="AF136" s="401"/>
       <c r="AG136" s="50"/>
       <c r="AH136" s="50"/>
       <c r="AI136" s="50"/>
@@ -11403,13 +11421,13 @@
       <c r="AK136" s="50"/>
       <c r="AL136" s="50"/>
       <c r="AM136" s="31"/>
-      <c r="AN136" s="407"/>
-      <c r="AO136" s="408"/>
-      <c r="AP136" s="408"/>
-      <c r="AQ136" s="408"/>
-      <c r="AR136" s="408"/>
-      <c r="AS136" s="408"/>
-      <c r="AT136" s="409"/>
+      <c r="AN136" s="408"/>
+      <c r="AO136" s="409"/>
+      <c r="AP136" s="409"/>
+      <c r="AQ136" s="409"/>
+      <c r="AR136" s="409"/>
+      <c r="AS136" s="409"/>
+      <c r="AT136" s="410"/>
       <c r="AU136" s="14"/>
       <c r="AZ136" s="56">
         <v>59200000</v>
@@ -11417,20 +11435,20 @@
     </row>
     <row r="137" spans="1:62" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A137" s="13"/>
-      <c r="B137" s="397" t="s">
+      <c r="B137" s="398" t="s">
         <v>63</v>
       </c>
-      <c r="C137" s="397"/>
-      <c r="D137" s="397"/>
-      <c r="E137" s="397"/>
-      <c r="F137" s="397"/>
-      <c r="G137" s="397"/>
-      <c r="H137" s="397"/>
-      <c r="I137" s="397"/>
-      <c r="J137" s="397"/>
-      <c r="K137" s="397"/>
+      <c r="C137" s="398"/>
+      <c r="D137" s="398"/>
+      <c r="E137" s="398"/>
+      <c r="F137" s="398"/>
+      <c r="G137" s="398"/>
+      <c r="H137" s="398"/>
+      <c r="I137" s="398"/>
+      <c r="J137" s="398"/>
+      <c r="K137" s="398"/>
       <c r="L137" s="155" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="M137" s="155"/>
       <c r="N137" s="155"/>
@@ -11452,10 +11470,10 @@
       <c r="AB137" s="55"/>
       <c r="AC137" s="55"/>
       <c r="AD137" s="31"/>
-      <c r="AE137" s="399" t="s">
-        <v>136</v>
-      </c>
-      <c r="AF137" s="400"/>
+      <c r="AE137" s="400" t="s">
+        <v>134</v>
+      </c>
+      <c r="AF137" s="401"/>
       <c r="AG137" s="50"/>
       <c r="AH137" s="50"/>
       <c r="AI137" s="50"/>
@@ -11463,13 +11481,13 @@
       <c r="AK137" s="50"/>
       <c r="AL137" s="50"/>
       <c r="AM137" s="31"/>
-      <c r="AN137" s="410"/>
-      <c r="AO137" s="411"/>
-      <c r="AP137" s="411"/>
-      <c r="AQ137" s="411"/>
-      <c r="AR137" s="411"/>
-      <c r="AS137" s="411"/>
-      <c r="AT137" s="412"/>
+      <c r="AN137" s="411"/>
+      <c r="AO137" s="412"/>
+      <c r="AP137" s="412"/>
+      <c r="AQ137" s="412"/>
+      <c r="AR137" s="412"/>
+      <c r="AS137" s="412"/>
+      <c r="AT137" s="413"/>
       <c r="AU137" s="14"/>
       <c r="AZ137" s="56">
         <f>+AZ136/1.19</f>
@@ -11633,152 +11651,152 @@
     </row>
     <row r="142" spans="1:62" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A142" s="13"/>
-      <c r="B142" s="396" t="s">
+      <c r="B142" s="397" t="s">
         <v>99</v>
       </c>
-      <c r="C142" s="396"/>
-      <c r="D142" s="396"/>
-      <c r="E142" s="396"/>
-      <c r="F142" s="396"/>
-      <c r="G142" s="396"/>
-      <c r="H142" s="396"/>
-      <c r="I142" s="396"/>
-      <c r="J142" s="396"/>
-      <c r="K142" s="396"/>
-      <c r="L142" s="396"/>
-      <c r="M142" s="396"/>
-      <c r="N142" s="396"/>
-      <c r="O142" s="396"/>
-      <c r="P142" s="396"/>
-      <c r="Q142" s="396"/>
-      <c r="R142" s="396"/>
-      <c r="S142" s="396"/>
-      <c r="T142" s="396"/>
-      <c r="U142" s="396"/>
-      <c r="V142" s="396"/>
-      <c r="W142" s="396"/>
-      <c r="X142" s="396"/>
-      <c r="Y142" s="396"/>
+      <c r="C142" s="397"/>
+      <c r="D142" s="397"/>
+      <c r="E142" s="397"/>
+      <c r="F142" s="397"/>
+      <c r="G142" s="397"/>
+      <c r="H142" s="397"/>
+      <c r="I142" s="397"/>
+      <c r="J142" s="397"/>
+      <c r="K142" s="397"/>
+      <c r="L142" s="397"/>
+      <c r="M142" s="397"/>
+      <c r="N142" s="397"/>
+      <c r="O142" s="397"/>
+      <c r="P142" s="397"/>
+      <c r="Q142" s="397"/>
+      <c r="R142" s="397"/>
+      <c r="S142" s="397"/>
+      <c r="T142" s="397"/>
+      <c r="U142" s="397"/>
+      <c r="V142" s="397"/>
+      <c r="W142" s="397"/>
+      <c r="X142" s="397"/>
+      <c r="Y142" s="397"/>
       <c r="Z142" s="1"/>
       <c r="AA142" s="1"/>
       <c r="AB142" s="1"/>
       <c r="AC142" s="4"/>
-      <c r="AD142" s="395" t="s">
+      <c r="AD142" s="396" t="s">
         <v>55</v>
       </c>
-      <c r="AE142" s="395"/>
-      <c r="AF142" s="395"/>
-      <c r="AG142" s="395"/>
-      <c r="AH142" s="395"/>
-      <c r="AI142" s="395"/>
-      <c r="AJ142" s="395"/>
-      <c r="AK142" s="395"/>
-      <c r="AL142" s="395"/>
-      <c r="AM142" s="395"/>
-      <c r="AN142" s="395"/>
-      <c r="AO142" s="395"/>
-      <c r="AP142" s="395"/>
-      <c r="AQ142" s="395"/>
-      <c r="AR142" s="395"/>
-      <c r="AS142" s="395"/>
+      <c r="AE142" s="396"/>
+      <c r="AF142" s="396"/>
+      <c r="AG142" s="396"/>
+      <c r="AH142" s="396"/>
+      <c r="AI142" s="396"/>
+      <c r="AJ142" s="396"/>
+      <c r="AK142" s="396"/>
+      <c r="AL142" s="396"/>
+      <c r="AM142" s="396"/>
+      <c r="AN142" s="396"/>
+      <c r="AO142" s="396"/>
+      <c r="AP142" s="396"/>
+      <c r="AQ142" s="396"/>
+      <c r="AR142" s="396"/>
+      <c r="AS142" s="396"/>
       <c r="AT142" s="25"/>
       <c r="AU142" s="14"/>
     </row>
     <row r="143" spans="1:62" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="13"/>
-      <c r="B143" s="396"/>
-      <c r="C143" s="396"/>
-      <c r="D143" s="396"/>
-      <c r="E143" s="396"/>
-      <c r="F143" s="396"/>
-      <c r="G143" s="396"/>
-      <c r="H143" s="396"/>
-      <c r="I143" s="396"/>
-      <c r="J143" s="396"/>
-      <c r="K143" s="396"/>
-      <c r="L143" s="396"/>
-      <c r="M143" s="396"/>
-      <c r="N143" s="396"/>
-      <c r="O143" s="396"/>
-      <c r="P143" s="396"/>
-      <c r="Q143" s="396"/>
-      <c r="R143" s="396"/>
-      <c r="S143" s="396"/>
-      <c r="T143" s="396"/>
-      <c r="U143" s="396"/>
-      <c r="V143" s="396"/>
-      <c r="W143" s="396"/>
-      <c r="X143" s="396"/>
-      <c r="Y143" s="396"/>
+      <c r="B143" s="397"/>
+      <c r="C143" s="397"/>
+      <c r="D143" s="397"/>
+      <c r="E143" s="397"/>
+      <c r="F143" s="397"/>
+      <c r="G143" s="397"/>
+      <c r="H143" s="397"/>
+      <c r="I143" s="397"/>
+      <c r="J143" s="397"/>
+      <c r="K143" s="397"/>
+      <c r="L143" s="397"/>
+      <c r="M143" s="397"/>
+      <c r="N143" s="397"/>
+      <c r="O143" s="397"/>
+      <c r="P143" s="397"/>
+      <c r="Q143" s="397"/>
+      <c r="R143" s="397"/>
+      <c r="S143" s="397"/>
+      <c r="T143" s="397"/>
+      <c r="U143" s="397"/>
+      <c r="V143" s="397"/>
+      <c r="W143" s="397"/>
+      <c r="X143" s="397"/>
+      <c r="Y143" s="397"/>
       <c r="Z143" s="1"/>
       <c r="AA143" s="1"/>
       <c r="AB143" s="2"/>
       <c r="AC143" s="4"/>
-      <c r="AD143" s="395"/>
-      <c r="AE143" s="395"/>
-      <c r="AF143" s="395"/>
-      <c r="AG143" s="395"/>
-      <c r="AH143" s="395"/>
-      <c r="AI143" s="395"/>
-      <c r="AJ143" s="395"/>
-      <c r="AK143" s="395"/>
-      <c r="AL143" s="395"/>
-      <c r="AM143" s="395"/>
-      <c r="AN143" s="395"/>
-      <c r="AO143" s="395"/>
-      <c r="AP143" s="395"/>
-      <c r="AQ143" s="395"/>
-      <c r="AR143" s="395"/>
-      <c r="AS143" s="395"/>
+      <c r="AD143" s="396"/>
+      <c r="AE143" s="396"/>
+      <c r="AF143" s="396"/>
+      <c r="AG143" s="396"/>
+      <c r="AH143" s="396"/>
+      <c r="AI143" s="396"/>
+      <c r="AJ143" s="396"/>
+      <c r="AK143" s="396"/>
+      <c r="AL143" s="396"/>
+      <c r="AM143" s="396"/>
+      <c r="AN143" s="396"/>
+      <c r="AO143" s="396"/>
+      <c r="AP143" s="396"/>
+      <c r="AQ143" s="396"/>
+      <c r="AR143" s="396"/>
+      <c r="AS143" s="396"/>
       <c r="AT143" s="25"/>
       <c r="AU143" s="14"/>
     </row>
     <row r="144" spans="1:62" ht="11.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A144" s="13"/>
-      <c r="B144" s="396"/>
-      <c r="C144" s="396"/>
-      <c r="D144" s="396"/>
-      <c r="E144" s="396"/>
-      <c r="F144" s="396"/>
-      <c r="G144" s="396"/>
-      <c r="H144" s="396"/>
-      <c r="I144" s="396"/>
-      <c r="J144" s="396"/>
-      <c r="K144" s="396"/>
-      <c r="L144" s="396"/>
-      <c r="M144" s="396"/>
-      <c r="N144" s="396"/>
-      <c r="O144" s="396"/>
-      <c r="P144" s="396"/>
-      <c r="Q144" s="396"/>
-      <c r="R144" s="396"/>
-      <c r="S144" s="396"/>
-      <c r="T144" s="396"/>
-      <c r="U144" s="396"/>
-      <c r="V144" s="396"/>
-      <c r="W144" s="396"/>
-      <c r="X144" s="396"/>
-      <c r="Y144" s="396"/>
+      <c r="B144" s="397"/>
+      <c r="C144" s="397"/>
+      <c r="D144" s="397"/>
+      <c r="E144" s="397"/>
+      <c r="F144" s="397"/>
+      <c r="G144" s="397"/>
+      <c r="H144" s="397"/>
+      <c r="I144" s="397"/>
+      <c r="J144" s="397"/>
+      <c r="K144" s="397"/>
+      <c r="L144" s="397"/>
+      <c r="M144" s="397"/>
+      <c r="N144" s="397"/>
+      <c r="O144" s="397"/>
+      <c r="P144" s="397"/>
+      <c r="Q144" s="397"/>
+      <c r="R144" s="397"/>
+      <c r="S144" s="397"/>
+      <c r="T144" s="397"/>
+      <c r="U144" s="397"/>
+      <c r="V144" s="397"/>
+      <c r="W144" s="397"/>
+      <c r="X144" s="397"/>
+      <c r="Y144" s="397"/>
       <c r="Z144" s="1"/>
       <c r="AA144" s="1"/>
       <c r="AB144" s="2"/>
       <c r="AC144" s="4"/>
-      <c r="AD144" s="395"/>
-      <c r="AE144" s="395"/>
-      <c r="AF144" s="395"/>
-      <c r="AG144" s="395"/>
-      <c r="AH144" s="395"/>
-      <c r="AI144" s="395"/>
-      <c r="AJ144" s="395"/>
-      <c r="AK144" s="395"/>
-      <c r="AL144" s="395"/>
-      <c r="AM144" s="395"/>
-      <c r="AN144" s="395"/>
-      <c r="AO144" s="395"/>
-      <c r="AP144" s="395"/>
-      <c r="AQ144" s="395"/>
-      <c r="AR144" s="395"/>
-      <c r="AS144" s="395"/>
+      <c r="AD144" s="396"/>
+      <c r="AE144" s="396"/>
+      <c r="AF144" s="396"/>
+      <c r="AG144" s="396"/>
+      <c r="AH144" s="396"/>
+      <c r="AI144" s="396"/>
+      <c r="AJ144" s="396"/>
+      <c r="AK144" s="396"/>
+      <c r="AL144" s="396"/>
+      <c r="AM144" s="396"/>
+      <c r="AN144" s="396"/>
+      <c r="AO144" s="396"/>
+      <c r="AP144" s="396"/>
+      <c r="AQ144" s="396"/>
+      <c r="AR144" s="396"/>
+      <c r="AS144" s="396"/>
       <c r="AT144" s="25"/>
       <c r="AU144" s="14"/>
       <c r="BJ144" s="3" t="s">
@@ -11787,130 +11805,130 @@
     </row>
     <row r="145" spans="1:47" s="31" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A145" s="29"/>
-      <c r="B145" s="396"/>
-      <c r="C145" s="396"/>
-      <c r="D145" s="396"/>
-      <c r="E145" s="396"/>
-      <c r="F145" s="396"/>
-      <c r="G145" s="396"/>
-      <c r="H145" s="396"/>
-      <c r="I145" s="396"/>
-      <c r="J145" s="396"/>
-      <c r="K145" s="396"/>
-      <c r="L145" s="396"/>
-      <c r="M145" s="396"/>
-      <c r="N145" s="396"/>
-      <c r="O145" s="396"/>
-      <c r="P145" s="396"/>
-      <c r="Q145" s="396"/>
-      <c r="R145" s="396"/>
-      <c r="S145" s="396"/>
-      <c r="T145" s="396"/>
-      <c r="U145" s="396"/>
-      <c r="V145" s="396"/>
-      <c r="W145" s="396"/>
-      <c r="X145" s="396"/>
-      <c r="Y145" s="396"/>
+      <c r="B145" s="397"/>
+      <c r="C145" s="397"/>
+      <c r="D145" s="397"/>
+      <c r="E145" s="397"/>
+      <c r="F145" s="397"/>
+      <c r="G145" s="397"/>
+      <c r="H145" s="397"/>
+      <c r="I145" s="397"/>
+      <c r="J145" s="397"/>
+      <c r="K145" s="397"/>
+      <c r="L145" s="397"/>
+      <c r="M145" s="397"/>
+      <c r="N145" s="397"/>
+      <c r="O145" s="397"/>
+      <c r="P145" s="397"/>
+      <c r="Q145" s="397"/>
+      <c r="R145" s="397"/>
+      <c r="S145" s="397"/>
+      <c r="T145" s="397"/>
+      <c r="U145" s="397"/>
+      <c r="V145" s="397"/>
+      <c r="W145" s="397"/>
+      <c r="X145" s="397"/>
+      <c r="Y145" s="397"/>
       <c r="Z145" s="1"/>
       <c r="AA145" s="1"/>
       <c r="AB145" s="2"/>
       <c r="AC145" s="4"/>
-      <c r="AD145" s="395"/>
-      <c r="AE145" s="395"/>
-      <c r="AF145" s="395"/>
-      <c r="AG145" s="395"/>
-      <c r="AH145" s="395"/>
-      <c r="AI145" s="395"/>
-      <c r="AJ145" s="395"/>
-      <c r="AK145" s="395"/>
-      <c r="AL145" s="395"/>
-      <c r="AM145" s="395"/>
-      <c r="AN145" s="395"/>
-      <c r="AO145" s="395"/>
-      <c r="AP145" s="395"/>
-      <c r="AQ145" s="395"/>
-      <c r="AR145" s="395"/>
-      <c r="AS145" s="395"/>
+      <c r="AD145" s="396"/>
+      <c r="AE145" s="396"/>
+      <c r="AF145" s="396"/>
+      <c r="AG145" s="396"/>
+      <c r="AH145" s="396"/>
+      <c r="AI145" s="396"/>
+      <c r="AJ145" s="396"/>
+      <c r="AK145" s="396"/>
+      <c r="AL145" s="396"/>
+      <c r="AM145" s="396"/>
+      <c r="AN145" s="396"/>
+      <c r="AO145" s="396"/>
+      <c r="AP145" s="396"/>
+      <c r="AQ145" s="396"/>
+      <c r="AR145" s="396"/>
+      <c r="AS145" s="396"/>
       <c r="AT145" s="25"/>
       <c r="AU145" s="30"/>
     </row>
     <row r="146" spans="1:47" s="31" customFormat="1" ht="12.65" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A146" s="29"/>
-      <c r="B146" s="396"/>
-      <c r="C146" s="396"/>
-      <c r="D146" s="396"/>
-      <c r="E146" s="396"/>
-      <c r="F146" s="396"/>
-      <c r="G146" s="396"/>
-      <c r="H146" s="396"/>
-      <c r="I146" s="396"/>
-      <c r="J146" s="396"/>
-      <c r="K146" s="396"/>
-      <c r="L146" s="396"/>
-      <c r="M146" s="396"/>
-      <c r="N146" s="396"/>
-      <c r="O146" s="396"/>
-      <c r="P146" s="396"/>
-      <c r="Q146" s="396"/>
-      <c r="R146" s="396"/>
-      <c r="S146" s="396"/>
-      <c r="T146" s="396"/>
-      <c r="U146" s="396"/>
-      <c r="V146" s="396"/>
-      <c r="W146" s="396"/>
-      <c r="X146" s="396"/>
-      <c r="Y146" s="396"/>
+      <c r="B146" s="397"/>
+      <c r="C146" s="397"/>
+      <c r="D146" s="397"/>
+      <c r="E146" s="397"/>
+      <c r="F146" s="397"/>
+      <c r="G146" s="397"/>
+      <c r="H146" s="397"/>
+      <c r="I146" s="397"/>
+      <c r="J146" s="397"/>
+      <c r="K146" s="397"/>
+      <c r="L146" s="397"/>
+      <c r="M146" s="397"/>
+      <c r="N146" s="397"/>
+      <c r="O146" s="397"/>
+      <c r="P146" s="397"/>
+      <c r="Q146" s="397"/>
+      <c r="R146" s="397"/>
+      <c r="S146" s="397"/>
+      <c r="T146" s="397"/>
+      <c r="U146" s="397"/>
+      <c r="V146" s="397"/>
+      <c r="W146" s="397"/>
+      <c r="X146" s="397"/>
+      <c r="Y146" s="397"/>
       <c r="Z146" s="1"/>
       <c r="AA146" s="1"/>
       <c r="AB146" s="2"/>
       <c r="AC146" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="AD146" s="398"/>
-      <c r="AE146" s="398"/>
-      <c r="AF146" s="398"/>
-      <c r="AG146" s="398"/>
-      <c r="AH146" s="398"/>
-      <c r="AI146" s="398"/>
-      <c r="AJ146" s="398"/>
-      <c r="AK146" s="398"/>
-      <c r="AL146" s="398"/>
-      <c r="AM146" s="398"/>
-      <c r="AN146" s="398"/>
-      <c r="AO146" s="398"/>
-      <c r="AP146" s="398"/>
-      <c r="AQ146" s="398"/>
-      <c r="AR146" s="398"/>
-      <c r="AS146" s="398"/>
+      <c r="AD146" s="399"/>
+      <c r="AE146" s="399"/>
+      <c r="AF146" s="399"/>
+      <c r="AG146" s="399"/>
+      <c r="AH146" s="399"/>
+      <c r="AI146" s="399"/>
+      <c r="AJ146" s="399"/>
+      <c r="AK146" s="399"/>
+      <c r="AL146" s="399"/>
+      <c r="AM146" s="399"/>
+      <c r="AN146" s="399"/>
+      <c r="AO146" s="399"/>
+      <c r="AP146" s="399"/>
+      <c r="AQ146" s="399"/>
+      <c r="AR146" s="399"/>
+      <c r="AS146" s="399"/>
       <c r="AT146" s="25"/>
       <c r="AU146" s="30"/>
     </row>
     <row r="147" spans="1:47" s="31" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A147" s="29"/>
-      <c r="B147" s="396"/>
-      <c r="C147" s="396"/>
-      <c r="D147" s="396"/>
-      <c r="E147" s="396"/>
-      <c r="F147" s="396"/>
-      <c r="G147" s="396"/>
-      <c r="H147" s="396"/>
-      <c r="I147" s="396"/>
-      <c r="J147" s="396"/>
-      <c r="K147" s="396"/>
-      <c r="L147" s="396"/>
-      <c r="M147" s="396"/>
-      <c r="N147" s="396"/>
-      <c r="O147" s="396"/>
-      <c r="P147" s="396"/>
-      <c r="Q147" s="396"/>
-      <c r="R147" s="396"/>
-      <c r="S147" s="396"/>
-      <c r="T147" s="396"/>
-      <c r="U147" s="396"/>
-      <c r="V147" s="396"/>
-      <c r="W147" s="396"/>
-      <c r="X147" s="396"/>
-      <c r="Y147" s="396"/>
+      <c r="B147" s="397"/>
+      <c r="C147" s="397"/>
+      <c r="D147" s="397"/>
+      <c r="E147" s="397"/>
+      <c r="F147" s="397"/>
+      <c r="G147" s="397"/>
+      <c r="H147" s="397"/>
+      <c r="I147" s="397"/>
+      <c r="J147" s="397"/>
+      <c r="K147" s="397"/>
+      <c r="L147" s="397"/>
+      <c r="M147" s="397"/>
+      <c r="N147" s="397"/>
+      <c r="O147" s="397"/>
+      <c r="P147" s="397"/>
+      <c r="Q147" s="397"/>
+      <c r="R147" s="397"/>
+      <c r="S147" s="397"/>
+      <c r="T147" s="397"/>
+      <c r="U147" s="397"/>
+      <c r="V147" s="397"/>
+      <c r="W147" s="397"/>
+      <c r="X147" s="397"/>
+      <c r="Y147" s="397"/>
       <c r="Z147" s="1"/>
       <c r="AA147" s="1"/>
       <c r="AB147" s="2"/>
@@ -11918,7 +11936,7 @@
         <v>40</v>
       </c>
       <c r="AD147" s="119" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="AE147" s="119"/>
       <c r="AF147" s="119"/>
@@ -11940,30 +11958,30 @@
     </row>
     <row r="148" spans="1:47" s="31" customFormat="1" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A148" s="29"/>
-      <c r="B148" s="396"/>
-      <c r="C148" s="396"/>
-      <c r="D148" s="396"/>
-      <c r="E148" s="396"/>
-      <c r="F148" s="396"/>
-      <c r="G148" s="396"/>
-      <c r="H148" s="396"/>
-      <c r="I148" s="396"/>
-      <c r="J148" s="396"/>
-      <c r="K148" s="396"/>
-      <c r="L148" s="396"/>
-      <c r="M148" s="396"/>
-      <c r="N148" s="396"/>
-      <c r="O148" s="396"/>
-      <c r="P148" s="396"/>
-      <c r="Q148" s="396"/>
-      <c r="R148" s="396"/>
-      <c r="S148" s="396"/>
-      <c r="T148" s="396"/>
-      <c r="U148" s="396"/>
-      <c r="V148" s="396"/>
-      <c r="W148" s="396"/>
-      <c r="X148" s="396"/>
-      <c r="Y148" s="396"/>
+      <c r="B148" s="397"/>
+      <c r="C148" s="397"/>
+      <c r="D148" s="397"/>
+      <c r="E148" s="397"/>
+      <c r="F148" s="397"/>
+      <c r="G148" s="397"/>
+      <c r="H148" s="397"/>
+      <c r="I148" s="397"/>
+      <c r="J148" s="397"/>
+      <c r="K148" s="397"/>
+      <c r="L148" s="397"/>
+      <c r="M148" s="397"/>
+      <c r="N148" s="397"/>
+      <c r="O148" s="397"/>
+      <c r="P148" s="397"/>
+      <c r="Q148" s="397"/>
+      <c r="R148" s="397"/>
+      <c r="S148" s="397"/>
+      <c r="T148" s="397"/>
+      <c r="U148" s="397"/>
+      <c r="V148" s="397"/>
+      <c r="W148" s="397"/>
+      <c r="X148" s="397"/>
+      <c r="Y148" s="397"/>
       <c r="Z148" s="1"/>
       <c r="AA148" s="1"/>
       <c r="AB148" s="2"/>
@@ -11971,7 +11989,7 @@
         <v>41</v>
       </c>
       <c r="AD148" s="119" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="AE148" s="119"/>
       <c r="AF148" s="119"/>
@@ -12023,7 +12041,7 @@
       <c r="AC149" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="AD149" s="413">
+      <c r="AD149" s="414">
         <v>46038</v>
       </c>
       <c r="AE149" s="119"/>
@@ -12192,208 +12210,208 @@
       <c r="AU152" s="44"/>
     </row>
     <row r="153" spans="1:47" ht="12.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A153" s="363" t="s">
+      <c r="A153" s="364" t="s">
         <v>76</v>
       </c>
-      <c r="B153" s="364"/>
-      <c r="C153" s="364"/>
-      <c r="D153" s="364"/>
-      <c r="E153" s="364"/>
-      <c r="F153" s="364"/>
-      <c r="G153" s="364"/>
-      <c r="H153" s="364"/>
-      <c r="I153" s="364"/>
-      <c r="J153" s="364"/>
-      <c r="K153" s="364"/>
-      <c r="L153" s="364"/>
-      <c r="M153" s="364"/>
-      <c r="N153" s="364"/>
-      <c r="O153" s="364"/>
-      <c r="P153" s="364"/>
-      <c r="Q153" s="364"/>
-      <c r="R153" s="364"/>
-      <c r="S153" s="364"/>
-      <c r="T153" s="364"/>
-      <c r="U153" s="364"/>
-      <c r="V153" s="364"/>
-      <c r="W153" s="364"/>
-      <c r="X153" s="364"/>
-      <c r="Y153" s="364"/>
-      <c r="Z153" s="364"/>
-      <c r="AA153" s="364"/>
-      <c r="AB153" s="364"/>
-      <c r="AC153" s="364"/>
-      <c r="AD153" s="364"/>
-      <c r="AE153" s="364"/>
-      <c r="AF153" s="364"/>
-      <c r="AG153" s="364"/>
-      <c r="AH153" s="364"/>
-      <c r="AI153" s="364"/>
-      <c r="AJ153" s="364"/>
-      <c r="AK153" s="364"/>
-      <c r="AL153" s="364"/>
-      <c r="AM153" s="364"/>
-      <c r="AN153" s="364"/>
-      <c r="AO153" s="364"/>
-      <c r="AP153" s="364"/>
-      <c r="AQ153" s="364"/>
-      <c r="AR153" s="364"/>
-      <c r="AS153" s="364"/>
-      <c r="AT153" s="364"/>
-      <c r="AU153" s="365"/>
+      <c r="B153" s="365"/>
+      <c r="C153" s="365"/>
+      <c r="D153" s="365"/>
+      <c r="E153" s="365"/>
+      <c r="F153" s="365"/>
+      <c r="G153" s="365"/>
+      <c r="H153" s="365"/>
+      <c r="I153" s="365"/>
+      <c r="J153" s="365"/>
+      <c r="K153" s="365"/>
+      <c r="L153" s="365"/>
+      <c r="M153" s="365"/>
+      <c r="N153" s="365"/>
+      <c r="O153" s="365"/>
+      <c r="P153" s="365"/>
+      <c r="Q153" s="365"/>
+      <c r="R153" s="365"/>
+      <c r="S153" s="365"/>
+      <c r="T153" s="365"/>
+      <c r="U153" s="365"/>
+      <c r="V153" s="365"/>
+      <c r="W153" s="365"/>
+      <c r="X153" s="365"/>
+      <c r="Y153" s="365"/>
+      <c r="Z153" s="365"/>
+      <c r="AA153" s="365"/>
+      <c r="AB153" s="365"/>
+      <c r="AC153" s="365"/>
+      <c r="AD153" s="365"/>
+      <c r="AE153" s="365"/>
+      <c r="AF153" s="365"/>
+      <c r="AG153" s="365"/>
+      <c r="AH153" s="365"/>
+      <c r="AI153" s="365"/>
+      <c r="AJ153" s="365"/>
+      <c r="AK153" s="365"/>
+      <c r="AL153" s="365"/>
+      <c r="AM153" s="365"/>
+      <c r="AN153" s="365"/>
+      <c r="AO153" s="365"/>
+      <c r="AP153" s="365"/>
+      <c r="AQ153" s="365"/>
+      <c r="AR153" s="365"/>
+      <c r="AS153" s="365"/>
+      <c r="AT153" s="365"/>
+      <c r="AU153" s="366"/>
     </row>
     <row r="154" spans="1:47" ht="309.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A154" s="401" t="s">
+      <c r="A154" s="402" t="s">
         <v>83</v>
       </c>
-      <c r="B154" s="402"/>
-      <c r="C154" s="402"/>
-      <c r="D154" s="402"/>
-      <c r="E154" s="402"/>
-      <c r="F154" s="402"/>
-      <c r="G154" s="402"/>
-      <c r="H154" s="402"/>
-      <c r="I154" s="402"/>
-      <c r="J154" s="402"/>
-      <c r="K154" s="402"/>
-      <c r="L154" s="402"/>
-      <c r="M154" s="402"/>
-      <c r="N154" s="402"/>
-      <c r="O154" s="402"/>
-      <c r="P154" s="402"/>
-      <c r="Q154" s="402"/>
-      <c r="R154" s="402"/>
-      <c r="S154" s="402"/>
-      <c r="T154" s="402"/>
-      <c r="U154" s="402"/>
-      <c r="V154" s="402"/>
-      <c r="W154" s="402"/>
-      <c r="X154" s="402"/>
-      <c r="Y154" s="402"/>
-      <c r="Z154" s="402"/>
-      <c r="AA154" s="402"/>
-      <c r="AB154" s="402"/>
-      <c r="AC154" s="402"/>
-      <c r="AD154" s="402"/>
-      <c r="AE154" s="402"/>
-      <c r="AF154" s="402"/>
-      <c r="AG154" s="402"/>
-      <c r="AH154" s="402"/>
-      <c r="AI154" s="402"/>
-      <c r="AJ154" s="402"/>
-      <c r="AK154" s="402"/>
-      <c r="AL154" s="402"/>
-      <c r="AM154" s="402"/>
-      <c r="AN154" s="402"/>
-      <c r="AO154" s="402"/>
-      <c r="AP154" s="402"/>
-      <c r="AQ154" s="402"/>
-      <c r="AR154" s="402"/>
-      <c r="AS154" s="402"/>
-      <c r="AT154" s="402"/>
-      <c r="AU154" s="403"/>
+      <c r="B154" s="403"/>
+      <c r="C154" s="403"/>
+      <c r="D154" s="403"/>
+      <c r="E154" s="403"/>
+      <c r="F154" s="403"/>
+      <c r="G154" s="403"/>
+      <c r="H154" s="403"/>
+      <c r="I154" s="403"/>
+      <c r="J154" s="403"/>
+      <c r="K154" s="403"/>
+      <c r="L154" s="403"/>
+      <c r="M154" s="403"/>
+      <c r="N154" s="403"/>
+      <c r="O154" s="403"/>
+      <c r="P154" s="403"/>
+      <c r="Q154" s="403"/>
+      <c r="R154" s="403"/>
+      <c r="S154" s="403"/>
+      <c r="T154" s="403"/>
+      <c r="U154" s="403"/>
+      <c r="V154" s="403"/>
+      <c r="W154" s="403"/>
+      <c r="X154" s="403"/>
+      <c r="Y154" s="403"/>
+      <c r="Z154" s="403"/>
+      <c r="AA154" s="403"/>
+      <c r="AB154" s="403"/>
+      <c r="AC154" s="403"/>
+      <c r="AD154" s="403"/>
+      <c r="AE154" s="403"/>
+      <c r="AF154" s="403"/>
+      <c r="AG154" s="403"/>
+      <c r="AH154" s="403"/>
+      <c r="AI154" s="403"/>
+      <c r="AJ154" s="403"/>
+      <c r="AK154" s="403"/>
+      <c r="AL154" s="403"/>
+      <c r="AM154" s="403"/>
+      <c r="AN154" s="403"/>
+      <c r="AO154" s="403"/>
+      <c r="AP154" s="403"/>
+      <c r="AQ154" s="403"/>
+      <c r="AR154" s="403"/>
+      <c r="AS154" s="403"/>
+      <c r="AT154" s="403"/>
+      <c r="AU154" s="404"/>
     </row>
     <row r="155" spans="1:47" ht="246.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A155" s="414" t="s">
+      <c r="A155" s="415" t="s">
         <v>92</v>
       </c>
-      <c r="B155" s="396"/>
-      <c r="C155" s="396"/>
-      <c r="D155" s="396"/>
-      <c r="E155" s="396"/>
-      <c r="F155" s="396"/>
-      <c r="G155" s="396"/>
-      <c r="H155" s="396"/>
-      <c r="I155" s="396"/>
-      <c r="J155" s="396"/>
-      <c r="K155" s="396"/>
-      <c r="L155" s="396"/>
-      <c r="M155" s="396"/>
-      <c r="N155" s="396"/>
-      <c r="O155" s="396"/>
-      <c r="P155" s="396"/>
-      <c r="Q155" s="396"/>
-      <c r="R155" s="396"/>
-      <c r="S155" s="396"/>
-      <c r="T155" s="396"/>
-      <c r="U155" s="396"/>
-      <c r="V155" s="396"/>
-      <c r="W155" s="396"/>
-      <c r="X155" s="396"/>
-      <c r="Y155" s="396"/>
-      <c r="Z155" s="396"/>
-      <c r="AA155" s="396"/>
-      <c r="AB155" s="396"/>
-      <c r="AC155" s="396"/>
-      <c r="AD155" s="396"/>
-      <c r="AE155" s="396"/>
-      <c r="AF155" s="396"/>
-      <c r="AG155" s="396"/>
-      <c r="AH155" s="396"/>
-      <c r="AI155" s="396"/>
-      <c r="AJ155" s="396"/>
-      <c r="AK155" s="396"/>
-      <c r="AL155" s="396"/>
-      <c r="AM155" s="396"/>
-      <c r="AN155" s="396"/>
-      <c r="AO155" s="396"/>
-      <c r="AP155" s="396"/>
-      <c r="AQ155" s="396"/>
-      <c r="AR155" s="396"/>
-      <c r="AS155" s="396"/>
-      <c r="AT155" s="396"/>
-      <c r="AU155" s="415"/>
+      <c r="B155" s="397"/>
+      <c r="C155" s="397"/>
+      <c r="D155" s="397"/>
+      <c r="E155" s="397"/>
+      <c r="F155" s="397"/>
+      <c r="G155" s="397"/>
+      <c r="H155" s="397"/>
+      <c r="I155" s="397"/>
+      <c r="J155" s="397"/>
+      <c r="K155" s="397"/>
+      <c r="L155" s="397"/>
+      <c r="M155" s="397"/>
+      <c r="N155" s="397"/>
+      <c r="O155" s="397"/>
+      <c r="P155" s="397"/>
+      <c r="Q155" s="397"/>
+      <c r="R155" s="397"/>
+      <c r="S155" s="397"/>
+      <c r="T155" s="397"/>
+      <c r="U155" s="397"/>
+      <c r="V155" s="397"/>
+      <c r="W155" s="397"/>
+      <c r="X155" s="397"/>
+      <c r="Y155" s="397"/>
+      <c r="Z155" s="397"/>
+      <c r="AA155" s="397"/>
+      <c r="AB155" s="397"/>
+      <c r="AC155" s="397"/>
+      <c r="AD155" s="397"/>
+      <c r="AE155" s="397"/>
+      <c r="AF155" s="397"/>
+      <c r="AG155" s="397"/>
+      <c r="AH155" s="397"/>
+      <c r="AI155" s="397"/>
+      <c r="AJ155" s="397"/>
+      <c r="AK155" s="397"/>
+      <c r="AL155" s="397"/>
+      <c r="AM155" s="397"/>
+      <c r="AN155" s="397"/>
+      <c r="AO155" s="397"/>
+      <c r="AP155" s="397"/>
+      <c r="AQ155" s="397"/>
+      <c r="AR155" s="397"/>
+      <c r="AS155" s="397"/>
+      <c r="AT155" s="397"/>
+      <c r="AU155" s="416"/>
     </row>
     <row r="156" spans="1:47" ht="110.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A156" s="392" t="s">
+      <c r="A156" s="393" t="s">
         <v>91</v>
       </c>
-      <c r="B156" s="393"/>
-      <c r="C156" s="393"/>
-      <c r="D156" s="393"/>
-      <c r="E156" s="393"/>
-      <c r="F156" s="393"/>
-      <c r="G156" s="393"/>
-      <c r="H156" s="393"/>
-      <c r="I156" s="393"/>
-      <c r="J156" s="393"/>
-      <c r="K156" s="393"/>
-      <c r="L156" s="393"/>
-      <c r="M156" s="393"/>
-      <c r="N156" s="393"/>
-      <c r="O156" s="393"/>
-      <c r="P156" s="393"/>
-      <c r="Q156" s="393"/>
-      <c r="R156" s="393"/>
-      <c r="S156" s="393"/>
-      <c r="T156" s="393"/>
-      <c r="U156" s="393"/>
-      <c r="V156" s="393"/>
-      <c r="W156" s="393"/>
-      <c r="X156" s="393"/>
-      <c r="Y156" s="393"/>
-      <c r="Z156" s="393"/>
-      <c r="AA156" s="393"/>
-      <c r="AB156" s="393"/>
-      <c r="AC156" s="393"/>
-      <c r="AD156" s="393"/>
-      <c r="AE156" s="393"/>
-      <c r="AF156" s="393"/>
-      <c r="AG156" s="393"/>
-      <c r="AH156" s="393"/>
-      <c r="AI156" s="393"/>
-      <c r="AJ156" s="393"/>
-      <c r="AK156" s="393"/>
-      <c r="AL156" s="393"/>
-      <c r="AM156" s="393"/>
-      <c r="AN156" s="393"/>
-      <c r="AO156" s="393"/>
-      <c r="AP156" s="393"/>
-      <c r="AQ156" s="393"/>
-      <c r="AR156" s="393"/>
-      <c r="AS156" s="393"/>
-      <c r="AT156" s="393"/>
-      <c r="AU156" s="394"/>
+      <c r="B156" s="394"/>
+      <c r="C156" s="394"/>
+      <c r="D156" s="394"/>
+      <c r="E156" s="394"/>
+      <c r="F156" s="394"/>
+      <c r="G156" s="394"/>
+      <c r="H156" s="394"/>
+      <c r="I156" s="394"/>
+      <c r="J156" s="394"/>
+      <c r="K156" s="394"/>
+      <c r="L156" s="394"/>
+      <c r="M156" s="394"/>
+      <c r="N156" s="394"/>
+      <c r="O156" s="394"/>
+      <c r="P156" s="394"/>
+      <c r="Q156" s="394"/>
+      <c r="R156" s="394"/>
+      <c r="S156" s="394"/>
+      <c r="T156" s="394"/>
+      <c r="U156" s="394"/>
+      <c r="V156" s="394"/>
+      <c r="W156" s="394"/>
+      <c r="X156" s="394"/>
+      <c r="Y156" s="394"/>
+      <c r="Z156" s="394"/>
+      <c r="AA156" s="394"/>
+      <c r="AB156" s="394"/>
+      <c r="AC156" s="394"/>
+      <c r="AD156" s="394"/>
+      <c r="AE156" s="394"/>
+      <c r="AF156" s="394"/>
+      <c r="AG156" s="394"/>
+      <c r="AH156" s="394"/>
+      <c r="AI156" s="394"/>
+      <c r="AJ156" s="394"/>
+      <c r="AK156" s="394"/>
+      <c r="AL156" s="394"/>
+      <c r="AM156" s="394"/>
+      <c r="AN156" s="394"/>
+      <c r="AO156" s="394"/>
+      <c r="AP156" s="394"/>
+      <c r="AQ156" s="394"/>
+      <c r="AR156" s="394"/>
+      <c r="AS156" s="394"/>
+      <c r="AT156" s="394"/>
+      <c r="AU156" s="395"/>
     </row>
   </sheetData>
   <mergeCells count="464">

</xml_diff>